<commit_message>
chore(data): sync FEB data 2026-04-06 00:17
</commit_message>
<xml_diff>
--- a/data/1FEB_25_26/clutch_lineups_25_26_1FEB.xlsx
+++ b/data/1FEB_25_26/clutch_lineups_25_26_1FEB.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X589"/>
+  <dimension ref="A1:X609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49942,6 +49942,1686 @@
         </is>
       </c>
     </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | J. PAUKSTÈ | J. PERIS CRESPO | J. ROUND | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>5</v>
+      </c>
+      <c r="E590" t="n">
+        <v>112</v>
+      </c>
+      <c r="F590" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="G590" t="n">
+        <v>3</v>
+      </c>
+      <c r="H590" t="n">
+        <v>2</v>
+      </c>
+      <c r="I590" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="J590" t="n">
+        <v>2</v>
+      </c>
+      <c r="K590" t="n">
+        <v>129.31</v>
+      </c>
+      <c r="L590" t="n">
+        <v>100</v>
+      </c>
+      <c r="M590" t="n">
+        <v>29.31</v>
+      </c>
+      <c r="N590" t="n">
+        <v>4</v>
+      </c>
+      <c r="O590" t="n">
+        <v>3</v>
+      </c>
+      <c r="P590" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q590" t="n">
+        <v>3</v>
+      </c>
+      <c r="R590" t="n">
+        <v>4</v>
+      </c>
+      <c r="S590" t="n">
+        <v>0</v>
+      </c>
+      <c r="T590" t="n">
+        <v>0</v>
+      </c>
+      <c r="U590" t="n">
+        <v>2</v>
+      </c>
+      <c r="V590" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W590" t="n">
+        <v>28</v>
+      </c>
+      <c r="X590" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | J. PERIS CRESPO | J. ROUND | J. VAN ZEGEREN | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>5</v>
+      </c>
+      <c r="E591" t="n">
+        <v>62</v>
+      </c>
+      <c r="F591" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G591" t="n">
+        <v>5</v>
+      </c>
+      <c r="H591" t="n">
+        <v>4</v>
+      </c>
+      <c r="I591" t="n">
+        <v>3</v>
+      </c>
+      <c r="J591" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="K591" t="n">
+        <v>166.67</v>
+      </c>
+      <c r="L591" t="n">
+        <v>103.09</v>
+      </c>
+      <c r="M591" t="n">
+        <v>63.57</v>
+      </c>
+      <c r="N591" t="n">
+        <v>2</v>
+      </c>
+      <c r="O591" t="n">
+        <v>0</v>
+      </c>
+      <c r="P591" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q591" t="n">
+        <v>0</v>
+      </c>
+      <c r="R591" t="n">
+        <v>2</v>
+      </c>
+      <c r="S591" t="n">
+        <v>2</v>
+      </c>
+      <c r="T591" t="n">
+        <v>1</v>
+      </c>
+      <c r="U591" t="n">
+        <v>0</v>
+      </c>
+      <c r="V591" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W591" t="n">
+        <v>28</v>
+      </c>
+      <c r="X591" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | J. PERIS CRESPO | J. VAN ZEGEREN | O. LO | T. NASPLER PERAIRE</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>5</v>
+      </c>
+      <c r="E592" t="n">
+        <v>43</v>
+      </c>
+      <c r="F592" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G592" t="n">
+        <v>0</v>
+      </c>
+      <c r="H592" t="n">
+        <v>0</v>
+      </c>
+      <c r="I592" t="n">
+        <v>1</v>
+      </c>
+      <c r="J592" t="n">
+        <v>1</v>
+      </c>
+      <c r="K592" t="n">
+        <v>0</v>
+      </c>
+      <c r="L592" t="n">
+        <v>0</v>
+      </c>
+      <c r="M592" t="n">
+        <v>0</v>
+      </c>
+      <c r="N592" t="n">
+        <v>3</v>
+      </c>
+      <c r="O592" t="n">
+        <v>0</v>
+      </c>
+      <c r="P592" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q592" t="n">
+        <v>2</v>
+      </c>
+      <c r="R592" t="n">
+        <v>1</v>
+      </c>
+      <c r="S592" t="n">
+        <v>0</v>
+      </c>
+      <c r="T592" t="n">
+        <v>0</v>
+      </c>
+      <c r="U592" t="n">
+        <v>0</v>
+      </c>
+      <c r="V592" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W592" t="n">
+        <v>28</v>
+      </c>
+      <c r="X592" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | J. ROUND | J. VAN ZEGEREN | O. LO | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>5</v>
+      </c>
+      <c r="E593" t="n">
+        <v>61</v>
+      </c>
+      <c r="F593" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G593" t="n">
+        <v>1</v>
+      </c>
+      <c r="H593" t="n">
+        <v>2</v>
+      </c>
+      <c r="I593" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J593" t="n">
+        <v>1</v>
+      </c>
+      <c r="K593" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="L593" t="n">
+        <v>200</v>
+      </c>
+      <c r="M593" t="n">
+        <v>-86.36</v>
+      </c>
+      <c r="N593" t="n">
+        <v>1</v>
+      </c>
+      <c r="O593" t="n">
+        <v>2</v>
+      </c>
+      <c r="P593" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q593" t="n">
+        <v>1</v>
+      </c>
+      <c r="R593" t="n">
+        <v>2</v>
+      </c>
+      <c r="S593" t="n">
+        <v>0</v>
+      </c>
+      <c r="T593" t="n">
+        <v>0</v>
+      </c>
+      <c r="U593" t="n">
+        <v>1</v>
+      </c>
+      <c r="V593" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W593" t="n">
+        <v>28</v>
+      </c>
+      <c r="X593" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>J. PERIS CRESPO | J. ROUND | O. LO | T. NASPLER PERAIRE | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>5</v>
+      </c>
+      <c r="E594" t="n">
+        <v>22</v>
+      </c>
+      <c r="F594" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G594" t="n">
+        <v>3</v>
+      </c>
+      <c r="H594" t="n">
+        <v>1</v>
+      </c>
+      <c r="I594" t="n">
+        <v>1</v>
+      </c>
+      <c r="J594" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="K594" t="n">
+        <v>300</v>
+      </c>
+      <c r="L594" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="M594" t="n">
+        <v>72.73</v>
+      </c>
+      <c r="N594" t="n">
+        <v>1</v>
+      </c>
+      <c r="O594" t="n">
+        <v>0</v>
+      </c>
+      <c r="P594" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q594" t="n">
+        <v>0</v>
+      </c>
+      <c r="R594" t="n">
+        <v>0</v>
+      </c>
+      <c r="S594" t="n">
+        <v>1</v>
+      </c>
+      <c r="T594" t="n">
+        <v>0</v>
+      </c>
+      <c r="U594" t="n">
+        <v>0</v>
+      </c>
+      <c r="V594" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W594" t="n">
+        <v>28</v>
+      </c>
+      <c r="X594" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>A. LIMA BRITO | D. MANCHON CRESPO | J. BELEMENE-DZABATOU | M. DIAZ | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>5</v>
+      </c>
+      <c r="E595" t="n">
+        <v>38</v>
+      </c>
+      <c r="F595" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G595" t="n">
+        <v>2</v>
+      </c>
+      <c r="H595" t="n">
+        <v>2</v>
+      </c>
+      <c r="I595" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J595" t="n">
+        <v>2</v>
+      </c>
+      <c r="K595" t="n">
+        <v>106.38</v>
+      </c>
+      <c r="L595" t="n">
+        <v>100</v>
+      </c>
+      <c r="M595" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="N595" t="n">
+        <v>1</v>
+      </c>
+      <c r="O595" t="n">
+        <v>2</v>
+      </c>
+      <c r="P595" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q595" t="n">
+        <v>0</v>
+      </c>
+      <c r="R595" t="n">
+        <v>1</v>
+      </c>
+      <c r="S595" t="n">
+        <v>0</v>
+      </c>
+      <c r="T595" t="n">
+        <v>1</v>
+      </c>
+      <c r="U595" t="n">
+        <v>0</v>
+      </c>
+      <c r="V595" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W595" t="n">
+        <v>28</v>
+      </c>
+      <c r="X595" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>A. LIMA BRITO | J. BELEMENE-DZABATOU | M. DIAZ | P. ALI | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>5</v>
+      </c>
+      <c r="E596" t="n">
+        <v>24</v>
+      </c>
+      <c r="F596" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G596" t="n">
+        <v>2</v>
+      </c>
+      <c r="H596" t="n">
+        <v>3</v>
+      </c>
+      <c r="I596" t="n">
+        <v>2</v>
+      </c>
+      <c r="J596" t="n">
+        <v>1</v>
+      </c>
+      <c r="K596" t="n">
+        <v>100</v>
+      </c>
+      <c r="L596" t="n">
+        <v>300</v>
+      </c>
+      <c r="M596" t="n">
+        <v>-200</v>
+      </c>
+      <c r="N596" t="n">
+        <v>1</v>
+      </c>
+      <c r="O596" t="n">
+        <v>0</v>
+      </c>
+      <c r="P596" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q596" t="n">
+        <v>0</v>
+      </c>
+      <c r="R596" t="n">
+        <v>1</v>
+      </c>
+      <c r="S596" t="n">
+        <v>0</v>
+      </c>
+      <c r="T596" t="n">
+        <v>0</v>
+      </c>
+      <c r="U596" t="n">
+        <v>0</v>
+      </c>
+      <c r="V596" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W596" t="n">
+        <v>28</v>
+      </c>
+      <c r="X596" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>D. MANCHON CRESPO | J. BELEMENE-DZABATOU | J. KASIBABU SHILALA | M. DIAZ | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D597" t="n">
+        <v>5</v>
+      </c>
+      <c r="E597" t="n">
+        <v>83</v>
+      </c>
+      <c r="F597" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="G597" t="n">
+        <v>2</v>
+      </c>
+      <c r="H597" t="n">
+        <v>2</v>
+      </c>
+      <c r="I597" t="n">
+        <v>1</v>
+      </c>
+      <c r="J597" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="K597" t="n">
+        <v>200</v>
+      </c>
+      <c r="L597" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="M597" t="n">
+        <v>130.56</v>
+      </c>
+      <c r="N597" t="n">
+        <v>3</v>
+      </c>
+      <c r="O597" t="n">
+        <v>0</v>
+      </c>
+      <c r="P597" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q597" t="n">
+        <v>2</v>
+      </c>
+      <c r="R597" t="n">
+        <v>4</v>
+      </c>
+      <c r="S597" t="n">
+        <v>2</v>
+      </c>
+      <c r="T597" t="n">
+        <v>0</v>
+      </c>
+      <c r="U597" t="n">
+        <v>2</v>
+      </c>
+      <c r="V597" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W597" t="n">
+        <v>28</v>
+      </c>
+      <c r="X597" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>J. BELEMENE-DZABATOU | J. KASIBABU SHILALA | M. DIAZ | P. ALI | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>5</v>
+      </c>
+      <c r="E598" t="n">
+        <v>155</v>
+      </c>
+      <c r="F598" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="G598" t="n">
+        <v>3</v>
+      </c>
+      <c r="H598" t="n">
+        <v>5</v>
+      </c>
+      <c r="I598" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="J598" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="K598" t="n">
+        <v>87.20999999999999</v>
+      </c>
+      <c r="L598" t="n">
+        <v>215.52</v>
+      </c>
+      <c r="M598" t="n">
+        <v>-128.31</v>
+      </c>
+      <c r="N598" t="n">
+        <v>4</v>
+      </c>
+      <c r="O598" t="n">
+        <v>1</v>
+      </c>
+      <c r="P598" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q598" t="n">
+        <v>1</v>
+      </c>
+      <c r="R598" t="n">
+        <v>5</v>
+      </c>
+      <c r="S598" t="n">
+        <v>3</v>
+      </c>
+      <c r="T598" t="n">
+        <v>0</v>
+      </c>
+      <c r="U598" t="n">
+        <v>4</v>
+      </c>
+      <c r="V598" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W598" t="n">
+        <v>28</v>
+      </c>
+      <c r="X598" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2486504</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | C. POLYNICE | I. RIVERA CARROLL | J. LOPEZ SANTANA | K. WEBSTER</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>5</v>
+      </c>
+      <c r="E599" t="n">
+        <v>134</v>
+      </c>
+      <c r="F599" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="G599" t="n">
+        <v>7</v>
+      </c>
+      <c r="H599" t="n">
+        <v>4</v>
+      </c>
+      <c r="I599" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="J599" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="K599" t="n">
+        <v>143.44</v>
+      </c>
+      <c r="L599" t="n">
+        <v>90.09</v>
+      </c>
+      <c r="M599" t="n">
+        <v>53.35</v>
+      </c>
+      <c r="N599" t="n">
+        <v>5</v>
+      </c>
+      <c r="O599" t="n">
+        <v>2</v>
+      </c>
+      <c r="P599" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q599" t="n">
+        <v>2</v>
+      </c>
+      <c r="R599" t="n">
+        <v>4</v>
+      </c>
+      <c r="S599" t="n">
+        <v>1</v>
+      </c>
+      <c r="T599" t="n">
+        <v>1</v>
+      </c>
+      <c r="U599" t="n">
+        <v>1</v>
+      </c>
+      <c r="V599" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W599" t="n">
+        <v>28</v>
+      </c>
+      <c r="X599" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2486504</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>J. GRANGER | L. GIOVANNETTI | O. SILVERIO GRULLON | P. GARINO GULLOTTA | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>5</v>
+      </c>
+      <c r="E600" t="n">
+        <v>17</v>
+      </c>
+      <c r="F600" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G600" t="n">
+        <v>2</v>
+      </c>
+      <c r="H600" t="n">
+        <v>0</v>
+      </c>
+      <c r="I600" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J600" t="n">
+        <v>0</v>
+      </c>
+      <c r="K600" t="n">
+        <v>138.89</v>
+      </c>
+      <c r="L600" t="n">
+        <v>0</v>
+      </c>
+      <c r="M600" t="n">
+        <v>0</v>
+      </c>
+      <c r="N600" t="n">
+        <v>2</v>
+      </c>
+      <c r="O600" t="n">
+        <v>1</v>
+      </c>
+      <c r="P600" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q600" t="n">
+        <v>1</v>
+      </c>
+      <c r="R600" t="n">
+        <v>0</v>
+      </c>
+      <c r="S600" t="n">
+        <v>0</v>
+      </c>
+      <c r="T600" t="n">
+        <v>1</v>
+      </c>
+      <c r="U600" t="n">
+        <v>1</v>
+      </c>
+      <c r="V600" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W600" t="n">
+        <v>28</v>
+      </c>
+      <c r="X600" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2486504</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>J. GRANGER | L. NWOGBO | O. SILVERIO GRULLON | P. GARINO GULLOTTA | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>5</v>
+      </c>
+      <c r="E601" t="n">
+        <v>91</v>
+      </c>
+      <c r="F601" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="G601" t="n">
+        <v>2</v>
+      </c>
+      <c r="H601" t="n">
+        <v>5</v>
+      </c>
+      <c r="I601" t="n">
+        <v>2</v>
+      </c>
+      <c r="J601" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="K601" t="n">
+        <v>100</v>
+      </c>
+      <c r="L601" t="n">
+        <v>128.87</v>
+      </c>
+      <c r="M601" t="n">
+        <v>-28.87</v>
+      </c>
+      <c r="N601" t="n">
+        <v>1</v>
+      </c>
+      <c r="O601" t="n">
+        <v>0</v>
+      </c>
+      <c r="P601" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q601" t="n">
+        <v>0</v>
+      </c>
+      <c r="R601" t="n">
+        <v>3</v>
+      </c>
+      <c r="S601" t="n">
+        <v>2</v>
+      </c>
+      <c r="T601" t="n">
+        <v>0</v>
+      </c>
+      <c r="U601" t="n">
+        <v>0</v>
+      </c>
+      <c r="V601" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W601" t="n">
+        <v>28</v>
+      </c>
+      <c r="X601" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2486504</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>J. GRANGER | O. SILVERIO GRULLON | P. GARINO GULLOTTA | R. STUMBRIS | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D602" t="n">
+        <v>5</v>
+      </c>
+      <c r="E602" t="n">
+        <v>26</v>
+      </c>
+      <c r="F602" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G602" t="n">
+        <v>0</v>
+      </c>
+      <c r="H602" t="n">
+        <v>2</v>
+      </c>
+      <c r="I602" t="n">
+        <v>1</v>
+      </c>
+      <c r="J602" t="n">
+        <v>1</v>
+      </c>
+      <c r="K602" t="n">
+        <v>0</v>
+      </c>
+      <c r="L602" t="n">
+        <v>200</v>
+      </c>
+      <c r="M602" t="n">
+        <v>-200</v>
+      </c>
+      <c r="N602" t="n">
+        <v>1</v>
+      </c>
+      <c r="O602" t="n">
+        <v>0</v>
+      </c>
+      <c r="P602" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q602" t="n">
+        <v>0</v>
+      </c>
+      <c r="R602" t="n">
+        <v>2</v>
+      </c>
+      <c r="S602" t="n">
+        <v>0</v>
+      </c>
+      <c r="T602" t="n">
+        <v>0</v>
+      </c>
+      <c r="U602" t="n">
+        <v>1</v>
+      </c>
+      <c r="V602" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W602" t="n">
+        <v>28</v>
+      </c>
+      <c r="X602" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>A. FAURE RIBES | D. DUSCAK | G. PARHAM II | J. ARIAS GONZALEZ | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D603" t="n">
+        <v>5</v>
+      </c>
+      <c r="E603" t="n">
+        <v>82</v>
+      </c>
+      <c r="F603" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="G603" t="n">
+        <v>0</v>
+      </c>
+      <c r="H603" t="n">
+        <v>2</v>
+      </c>
+      <c r="I603" t="n">
+        <v>1</v>
+      </c>
+      <c r="J603" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="K603" t="n">
+        <v>0</v>
+      </c>
+      <c r="L603" t="n">
+        <v>106.38</v>
+      </c>
+      <c r="M603" t="n">
+        <v>-106.38</v>
+      </c>
+      <c r="N603" t="n">
+        <v>2</v>
+      </c>
+      <c r="O603" t="n">
+        <v>0</v>
+      </c>
+      <c r="P603" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q603" t="n">
+        <v>1</v>
+      </c>
+      <c r="R603" t="n">
+        <v>2</v>
+      </c>
+      <c r="S603" t="n">
+        <v>2</v>
+      </c>
+      <c r="T603" t="n">
+        <v>0</v>
+      </c>
+      <c r="U603" t="n">
+        <v>1</v>
+      </c>
+      <c r="V603" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W603" t="n">
+        <v>28</v>
+      </c>
+      <c r="X603" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>A. FAURE RIBES | D. DUSCAK | G. PARHAM II | M. TOWNES VILLAR | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D604" t="n">
+        <v>5</v>
+      </c>
+      <c r="E604" t="n">
+        <v>44</v>
+      </c>
+      <c r="F604" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G604" t="n">
+        <v>2</v>
+      </c>
+      <c r="H604" t="n">
+        <v>4</v>
+      </c>
+      <c r="I604" t="n">
+        <v>2</v>
+      </c>
+      <c r="J604" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="K604" t="n">
+        <v>100</v>
+      </c>
+      <c r="L604" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="M604" t="n">
+        <v>-112.77</v>
+      </c>
+      <c r="N604" t="n">
+        <v>2</v>
+      </c>
+      <c r="O604" t="n">
+        <v>0</v>
+      </c>
+      <c r="P604" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q604" t="n">
+        <v>0</v>
+      </c>
+      <c r="R604" t="n">
+        <v>1</v>
+      </c>
+      <c r="S604" t="n">
+        <v>2</v>
+      </c>
+      <c r="T604" t="n">
+        <v>0</v>
+      </c>
+      <c r="U604" t="n">
+        <v>0</v>
+      </c>
+      <c r="V604" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W604" t="n">
+        <v>28</v>
+      </c>
+      <c r="X604" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>D. DUSCAK | G. PARHAM II | M. TOWNES VILLAR | R. COSIALLS BORRAS | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D605" t="n">
+        <v>5</v>
+      </c>
+      <c r="E605" t="n">
+        <v>90</v>
+      </c>
+      <c r="F605" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G605" t="n">
+        <v>2</v>
+      </c>
+      <c r="H605" t="n">
+        <v>4</v>
+      </c>
+      <c r="I605" t="n">
+        <v>3</v>
+      </c>
+      <c r="J605" t="n">
+        <v>2</v>
+      </c>
+      <c r="K605" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="L605" t="n">
+        <v>200</v>
+      </c>
+      <c r="M605" t="n">
+        <v>-133.33</v>
+      </c>
+      <c r="N605" t="n">
+        <v>3</v>
+      </c>
+      <c r="O605" t="n">
+        <v>0</v>
+      </c>
+      <c r="P605" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q605" t="n">
+        <v>0</v>
+      </c>
+      <c r="R605" t="n">
+        <v>2</v>
+      </c>
+      <c r="S605" t="n">
+        <v>0</v>
+      </c>
+      <c r="T605" t="n">
+        <v>0</v>
+      </c>
+      <c r="U605" t="n">
+        <v>0</v>
+      </c>
+      <c r="V605" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W605" t="n">
+        <v>28</v>
+      </c>
+      <c r="X605" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>F. NWAOKORIE | J. ARIAS GONZALEZ | M. TOWNES VILLAR | R. COSIALLS BORRAS | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D606" t="n">
+        <v>5</v>
+      </c>
+      <c r="E606" t="n">
+        <v>10</v>
+      </c>
+      <c r="F606" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G606" t="n">
+        <v>2</v>
+      </c>
+      <c r="H606" t="n">
+        <v>0</v>
+      </c>
+      <c r="I606" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="J606" t="n">
+        <v>1</v>
+      </c>
+      <c r="K606" t="n">
+        <v>0</v>
+      </c>
+      <c r="L606" t="n">
+        <v>0</v>
+      </c>
+      <c r="M606" t="n">
+        <v>0</v>
+      </c>
+      <c r="N606" t="n">
+        <v>0</v>
+      </c>
+      <c r="O606" t="n">
+        <v>2</v>
+      </c>
+      <c r="P606" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q606" t="n">
+        <v>1</v>
+      </c>
+      <c r="R606" t="n">
+        <v>1</v>
+      </c>
+      <c r="S606" t="n">
+        <v>0</v>
+      </c>
+      <c r="T606" t="n">
+        <v>0</v>
+      </c>
+      <c r="U606" t="n">
+        <v>0</v>
+      </c>
+      <c r="V606" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W606" t="n">
+        <v>28</v>
+      </c>
+      <c r="X606" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>A. JORDA RODRIGUEZ | D. GEU | J. BONE | K. LARSEN | M. TORRES CUEVAS</t>
+        </is>
+      </c>
+      <c r="D607" t="n">
+        <v>5</v>
+      </c>
+      <c r="E607" t="n">
+        <v>206</v>
+      </c>
+      <c r="F607" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="G607" t="n">
+        <v>10</v>
+      </c>
+      <c r="H607" t="n">
+        <v>4</v>
+      </c>
+      <c r="I607" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="J607" t="n">
+        <v>6</v>
+      </c>
+      <c r="K607" t="n">
+        <v>173.61</v>
+      </c>
+      <c r="L607" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="M607" t="n">
+        <v>106.94</v>
+      </c>
+      <c r="N607" t="n">
+        <v>5</v>
+      </c>
+      <c r="O607" t="n">
+        <v>4</v>
+      </c>
+      <c r="P607" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q607" t="n">
+        <v>1</v>
+      </c>
+      <c r="R607" t="n">
+        <v>7</v>
+      </c>
+      <c r="S607" t="n">
+        <v>0</v>
+      </c>
+      <c r="T607" t="n">
+        <v>0</v>
+      </c>
+      <c r="U607" t="n">
+        <v>1</v>
+      </c>
+      <c r="V607" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W607" t="n">
+        <v>28</v>
+      </c>
+      <c r="X607" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>A. JORDA RODRIGUEZ | D. GEU | J. BONE | M. TORRES CUEVAS | U. MENDICOTE RUBIO</t>
+        </is>
+      </c>
+      <c r="D608" t="n">
+        <v>5</v>
+      </c>
+      <c r="E608" t="n">
+        <v>10</v>
+      </c>
+      <c r="F608" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G608" t="n">
+        <v>0</v>
+      </c>
+      <c r="H608" t="n">
+        <v>0</v>
+      </c>
+      <c r="I608" t="n">
+        <v>0</v>
+      </c>
+      <c r="J608" t="n">
+        <v>0</v>
+      </c>
+      <c r="K608" t="n">
+        <v>0</v>
+      </c>
+      <c r="L608" t="n">
+        <v>0</v>
+      </c>
+      <c r="M608" t="n">
+        <v>0</v>
+      </c>
+      <c r="N608" t="n">
+        <v>0</v>
+      </c>
+      <c r="O608" t="n">
+        <v>0</v>
+      </c>
+      <c r="P608" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q608" t="n">
+        <v>0</v>
+      </c>
+      <c r="R608" t="n">
+        <v>0</v>
+      </c>
+      <c r="S608" t="n">
+        <v>0</v>
+      </c>
+      <c r="T608" t="n">
+        <v>0</v>
+      </c>
+      <c r="U608" t="n">
+        <v>0</v>
+      </c>
+      <c r="V608" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W608" t="n">
+        <v>28</v>
+      </c>
+      <c r="X608" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>A. JORDA RODRIGUEZ | J. BONE | J. MWEMA | K. LARSEN | M. TORRES CUEVAS</t>
+        </is>
+      </c>
+      <c r="D609" t="n">
+        <v>5</v>
+      </c>
+      <c r="E609" t="n">
+        <v>10</v>
+      </c>
+      <c r="F609" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G609" t="n">
+        <v>0</v>
+      </c>
+      <c r="H609" t="n">
+        <v>2</v>
+      </c>
+      <c r="I609" t="n">
+        <v>1</v>
+      </c>
+      <c r="J609" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="K609" t="n">
+        <v>0</v>
+      </c>
+      <c r="L609" t="n">
+        <v>0</v>
+      </c>
+      <c r="M609" t="n">
+        <v>0</v>
+      </c>
+      <c r="N609" t="n">
+        <v>1</v>
+      </c>
+      <c r="O609" t="n">
+        <v>0</v>
+      </c>
+      <c r="P609" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q609" t="n">
+        <v>0</v>
+      </c>
+      <c r="R609" t="n">
+        <v>0</v>
+      </c>
+      <c r="S609" t="n">
+        <v>2</v>
+      </c>
+      <c r="T609" t="n">
+        <v>0</v>
+      </c>
+      <c r="U609" t="n">
+        <v>1</v>
+      </c>
+      <c r="V609" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W609" t="n">
+        <v>28</v>
+      </c>
+      <c r="X609" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): sync FEB data 2026-04-13 13:19
</commit_message>
<xml_diff>
--- a/data/1FEB_25_26/clutch_lineups_25_26_1FEB.xlsx
+++ b/data/1FEB_25_26/clutch_lineups_25_26_1FEB.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X589"/>
+  <dimension ref="A1:X645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49942,6 +49942,4710 @@
         </is>
       </c>
     </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | J. PAUKSTÈ | J. PERIS CRESPO | J. ROUND | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>5</v>
+      </c>
+      <c r="E590" t="n">
+        <v>112</v>
+      </c>
+      <c r="F590" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="G590" t="n">
+        <v>3</v>
+      </c>
+      <c r="H590" t="n">
+        <v>2</v>
+      </c>
+      <c r="I590" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="J590" t="n">
+        <v>2</v>
+      </c>
+      <c r="K590" t="n">
+        <v>129.31</v>
+      </c>
+      <c r="L590" t="n">
+        <v>100</v>
+      </c>
+      <c r="M590" t="n">
+        <v>29.31</v>
+      </c>
+      <c r="N590" t="n">
+        <v>4</v>
+      </c>
+      <c r="O590" t="n">
+        <v>3</v>
+      </c>
+      <c r="P590" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q590" t="n">
+        <v>3</v>
+      </c>
+      <c r="R590" t="n">
+        <v>4</v>
+      </c>
+      <c r="S590" t="n">
+        <v>0</v>
+      </c>
+      <c r="T590" t="n">
+        <v>0</v>
+      </c>
+      <c r="U590" t="n">
+        <v>2</v>
+      </c>
+      <c r="V590" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W590" t="n">
+        <v>28</v>
+      </c>
+      <c r="X590" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | J. PERIS CRESPO | J. ROUND | J. VAN ZEGEREN | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>5</v>
+      </c>
+      <c r="E591" t="n">
+        <v>62</v>
+      </c>
+      <c r="F591" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G591" t="n">
+        <v>5</v>
+      </c>
+      <c r="H591" t="n">
+        <v>4</v>
+      </c>
+      <c r="I591" t="n">
+        <v>3</v>
+      </c>
+      <c r="J591" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="K591" t="n">
+        <v>166.67</v>
+      </c>
+      <c r="L591" t="n">
+        <v>103.09</v>
+      </c>
+      <c r="M591" t="n">
+        <v>63.57</v>
+      </c>
+      <c r="N591" t="n">
+        <v>2</v>
+      </c>
+      <c r="O591" t="n">
+        <v>0</v>
+      </c>
+      <c r="P591" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q591" t="n">
+        <v>0</v>
+      </c>
+      <c r="R591" t="n">
+        <v>2</v>
+      </c>
+      <c r="S591" t="n">
+        <v>2</v>
+      </c>
+      <c r="T591" t="n">
+        <v>1</v>
+      </c>
+      <c r="U591" t="n">
+        <v>0</v>
+      </c>
+      <c r="V591" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W591" t="n">
+        <v>28</v>
+      </c>
+      <c r="X591" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | J. PERIS CRESPO | J. VAN ZEGEREN | O. LO | T. NASPLER PERAIRE</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>5</v>
+      </c>
+      <c r="E592" t="n">
+        <v>43</v>
+      </c>
+      <c r="F592" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G592" t="n">
+        <v>0</v>
+      </c>
+      <c r="H592" t="n">
+        <v>0</v>
+      </c>
+      <c r="I592" t="n">
+        <v>1</v>
+      </c>
+      <c r="J592" t="n">
+        <v>1</v>
+      </c>
+      <c r="K592" t="n">
+        <v>0</v>
+      </c>
+      <c r="L592" t="n">
+        <v>0</v>
+      </c>
+      <c r="M592" t="n">
+        <v>0</v>
+      </c>
+      <c r="N592" t="n">
+        <v>3</v>
+      </c>
+      <c r="O592" t="n">
+        <v>0</v>
+      </c>
+      <c r="P592" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q592" t="n">
+        <v>2</v>
+      </c>
+      <c r="R592" t="n">
+        <v>1</v>
+      </c>
+      <c r="S592" t="n">
+        <v>0</v>
+      </c>
+      <c r="T592" t="n">
+        <v>0</v>
+      </c>
+      <c r="U592" t="n">
+        <v>0</v>
+      </c>
+      <c r="V592" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W592" t="n">
+        <v>28</v>
+      </c>
+      <c r="X592" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | J. ROUND | J. VAN ZEGEREN | O. LO | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>5</v>
+      </c>
+      <c r="E593" t="n">
+        <v>61</v>
+      </c>
+      <c r="F593" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G593" t="n">
+        <v>1</v>
+      </c>
+      <c r="H593" t="n">
+        <v>2</v>
+      </c>
+      <c r="I593" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J593" t="n">
+        <v>1</v>
+      </c>
+      <c r="K593" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="L593" t="n">
+        <v>200</v>
+      </c>
+      <c r="M593" t="n">
+        <v>-86.36</v>
+      </c>
+      <c r="N593" t="n">
+        <v>1</v>
+      </c>
+      <c r="O593" t="n">
+        <v>2</v>
+      </c>
+      <c r="P593" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q593" t="n">
+        <v>1</v>
+      </c>
+      <c r="R593" t="n">
+        <v>2</v>
+      </c>
+      <c r="S593" t="n">
+        <v>0</v>
+      </c>
+      <c r="T593" t="n">
+        <v>0</v>
+      </c>
+      <c r="U593" t="n">
+        <v>1</v>
+      </c>
+      <c r="V593" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W593" t="n">
+        <v>28</v>
+      </c>
+      <c r="X593" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>J. PERIS CRESPO | J. ROUND | O. LO | T. NASPLER PERAIRE | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>5</v>
+      </c>
+      <c r="E594" t="n">
+        <v>22</v>
+      </c>
+      <c r="F594" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G594" t="n">
+        <v>3</v>
+      </c>
+      <c r="H594" t="n">
+        <v>1</v>
+      </c>
+      <c r="I594" t="n">
+        <v>1</v>
+      </c>
+      <c r="J594" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="K594" t="n">
+        <v>300</v>
+      </c>
+      <c r="L594" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="M594" t="n">
+        <v>72.73</v>
+      </c>
+      <c r="N594" t="n">
+        <v>1</v>
+      </c>
+      <c r="O594" t="n">
+        <v>0</v>
+      </c>
+      <c r="P594" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q594" t="n">
+        <v>0</v>
+      </c>
+      <c r="R594" t="n">
+        <v>0</v>
+      </c>
+      <c r="S594" t="n">
+        <v>1</v>
+      </c>
+      <c r="T594" t="n">
+        <v>0</v>
+      </c>
+      <c r="U594" t="n">
+        <v>0</v>
+      </c>
+      <c r="V594" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W594" t="n">
+        <v>28</v>
+      </c>
+      <c r="X594" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>A. LIMA BRITO | D. MANCHON CRESPO | J. BELEMENE-DZABATOU | M. DIAZ | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>5</v>
+      </c>
+      <c r="E595" t="n">
+        <v>38</v>
+      </c>
+      <c r="F595" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G595" t="n">
+        <v>2</v>
+      </c>
+      <c r="H595" t="n">
+        <v>2</v>
+      </c>
+      <c r="I595" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J595" t="n">
+        <v>2</v>
+      </c>
+      <c r="K595" t="n">
+        <v>106.38</v>
+      </c>
+      <c r="L595" t="n">
+        <v>100</v>
+      </c>
+      <c r="M595" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="N595" t="n">
+        <v>1</v>
+      </c>
+      <c r="O595" t="n">
+        <v>2</v>
+      </c>
+      <c r="P595" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q595" t="n">
+        <v>0</v>
+      </c>
+      <c r="R595" t="n">
+        <v>1</v>
+      </c>
+      <c r="S595" t="n">
+        <v>0</v>
+      </c>
+      <c r="T595" t="n">
+        <v>1</v>
+      </c>
+      <c r="U595" t="n">
+        <v>0</v>
+      </c>
+      <c r="V595" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W595" t="n">
+        <v>28</v>
+      </c>
+      <c r="X595" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>A. LIMA BRITO | J. BELEMENE-DZABATOU | M. DIAZ | P. ALI | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>5</v>
+      </c>
+      <c r="E596" t="n">
+        <v>24</v>
+      </c>
+      <c r="F596" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G596" t="n">
+        <v>2</v>
+      </c>
+      <c r="H596" t="n">
+        <v>3</v>
+      </c>
+      <c r="I596" t="n">
+        <v>2</v>
+      </c>
+      <c r="J596" t="n">
+        <v>1</v>
+      </c>
+      <c r="K596" t="n">
+        <v>100</v>
+      </c>
+      <c r="L596" t="n">
+        <v>300</v>
+      </c>
+      <c r="M596" t="n">
+        <v>-200</v>
+      </c>
+      <c r="N596" t="n">
+        <v>1</v>
+      </c>
+      <c r="O596" t="n">
+        <v>0</v>
+      </c>
+      <c r="P596" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q596" t="n">
+        <v>0</v>
+      </c>
+      <c r="R596" t="n">
+        <v>1</v>
+      </c>
+      <c r="S596" t="n">
+        <v>0</v>
+      </c>
+      <c r="T596" t="n">
+        <v>0</v>
+      </c>
+      <c r="U596" t="n">
+        <v>0</v>
+      </c>
+      <c r="V596" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W596" t="n">
+        <v>28</v>
+      </c>
+      <c r="X596" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>D. MANCHON CRESPO | J. BELEMENE-DZABATOU | J. KASIBABU SHILALA | M. DIAZ | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D597" t="n">
+        <v>5</v>
+      </c>
+      <c r="E597" t="n">
+        <v>83</v>
+      </c>
+      <c r="F597" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="G597" t="n">
+        <v>2</v>
+      </c>
+      <c r="H597" t="n">
+        <v>2</v>
+      </c>
+      <c r="I597" t="n">
+        <v>1</v>
+      </c>
+      <c r="J597" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="K597" t="n">
+        <v>200</v>
+      </c>
+      <c r="L597" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="M597" t="n">
+        <v>130.56</v>
+      </c>
+      <c r="N597" t="n">
+        <v>3</v>
+      </c>
+      <c r="O597" t="n">
+        <v>0</v>
+      </c>
+      <c r="P597" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q597" t="n">
+        <v>2</v>
+      </c>
+      <c r="R597" t="n">
+        <v>4</v>
+      </c>
+      <c r="S597" t="n">
+        <v>2</v>
+      </c>
+      <c r="T597" t="n">
+        <v>0</v>
+      </c>
+      <c r="U597" t="n">
+        <v>2</v>
+      </c>
+      <c r="V597" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W597" t="n">
+        <v>28</v>
+      </c>
+      <c r="X597" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2486507</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>J. BELEMENE-DZABATOU | J. KASIBABU SHILALA | M. DIAZ | P. ALI | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>5</v>
+      </c>
+      <c r="E598" t="n">
+        <v>155</v>
+      </c>
+      <c r="F598" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="G598" t="n">
+        <v>3</v>
+      </c>
+      <c r="H598" t="n">
+        <v>5</v>
+      </c>
+      <c r="I598" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="J598" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="K598" t="n">
+        <v>87.20999999999999</v>
+      </c>
+      <c r="L598" t="n">
+        <v>215.52</v>
+      </c>
+      <c r="M598" t="n">
+        <v>-128.31</v>
+      </c>
+      <c r="N598" t="n">
+        <v>4</v>
+      </c>
+      <c r="O598" t="n">
+        <v>1</v>
+      </c>
+      <c r="P598" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q598" t="n">
+        <v>1</v>
+      </c>
+      <c r="R598" t="n">
+        <v>5</v>
+      </c>
+      <c r="S598" t="n">
+        <v>3</v>
+      </c>
+      <c r="T598" t="n">
+        <v>0</v>
+      </c>
+      <c r="U598" t="n">
+        <v>4</v>
+      </c>
+      <c r="V598" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W598" t="n">
+        <v>28</v>
+      </c>
+      <c r="X598" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2486504</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | C. POLYNICE | I. RIVERA CARROLL | J. LOPEZ SANTANA | K. WEBSTER</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>5</v>
+      </c>
+      <c r="E599" t="n">
+        <v>134</v>
+      </c>
+      <c r="F599" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="G599" t="n">
+        <v>7</v>
+      </c>
+      <c r="H599" t="n">
+        <v>4</v>
+      </c>
+      <c r="I599" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="J599" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="K599" t="n">
+        <v>143.44</v>
+      </c>
+      <c r="L599" t="n">
+        <v>90.09</v>
+      </c>
+      <c r="M599" t="n">
+        <v>53.35</v>
+      </c>
+      <c r="N599" t="n">
+        <v>5</v>
+      </c>
+      <c r="O599" t="n">
+        <v>2</v>
+      </c>
+      <c r="P599" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q599" t="n">
+        <v>2</v>
+      </c>
+      <c r="R599" t="n">
+        <v>4</v>
+      </c>
+      <c r="S599" t="n">
+        <v>1</v>
+      </c>
+      <c r="T599" t="n">
+        <v>1</v>
+      </c>
+      <c r="U599" t="n">
+        <v>1</v>
+      </c>
+      <c r="V599" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W599" t="n">
+        <v>28</v>
+      </c>
+      <c r="X599" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2486504</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>J. GRANGER | L. GIOVANNETTI | O. SILVERIO GRULLON | P. GARINO GULLOTTA | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>5</v>
+      </c>
+      <c r="E600" t="n">
+        <v>17</v>
+      </c>
+      <c r="F600" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G600" t="n">
+        <v>2</v>
+      </c>
+      <c r="H600" t="n">
+        <v>0</v>
+      </c>
+      <c r="I600" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J600" t="n">
+        <v>0</v>
+      </c>
+      <c r="K600" t="n">
+        <v>138.89</v>
+      </c>
+      <c r="L600" t="n">
+        <v>0</v>
+      </c>
+      <c r="M600" t="n">
+        <v>0</v>
+      </c>
+      <c r="N600" t="n">
+        <v>2</v>
+      </c>
+      <c r="O600" t="n">
+        <v>1</v>
+      </c>
+      <c r="P600" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q600" t="n">
+        <v>1</v>
+      </c>
+      <c r="R600" t="n">
+        <v>0</v>
+      </c>
+      <c r="S600" t="n">
+        <v>0</v>
+      </c>
+      <c r="T600" t="n">
+        <v>1</v>
+      </c>
+      <c r="U600" t="n">
+        <v>1</v>
+      </c>
+      <c r="V600" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W600" t="n">
+        <v>28</v>
+      </c>
+      <c r="X600" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2486504</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>J. GRANGER | L. NWOGBO | O. SILVERIO GRULLON | P. GARINO GULLOTTA | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>5</v>
+      </c>
+      <c r="E601" t="n">
+        <v>91</v>
+      </c>
+      <c r="F601" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="G601" t="n">
+        <v>2</v>
+      </c>
+      <c r="H601" t="n">
+        <v>5</v>
+      </c>
+      <c r="I601" t="n">
+        <v>2</v>
+      </c>
+      <c r="J601" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="K601" t="n">
+        <v>100</v>
+      </c>
+      <c r="L601" t="n">
+        <v>128.87</v>
+      </c>
+      <c r="M601" t="n">
+        <v>-28.87</v>
+      </c>
+      <c r="N601" t="n">
+        <v>1</v>
+      </c>
+      <c r="O601" t="n">
+        <v>0</v>
+      </c>
+      <c r="P601" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q601" t="n">
+        <v>0</v>
+      </c>
+      <c r="R601" t="n">
+        <v>3</v>
+      </c>
+      <c r="S601" t="n">
+        <v>2</v>
+      </c>
+      <c r="T601" t="n">
+        <v>0</v>
+      </c>
+      <c r="U601" t="n">
+        <v>0</v>
+      </c>
+      <c r="V601" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W601" t="n">
+        <v>28</v>
+      </c>
+      <c r="X601" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2486504</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>J. GRANGER | O. SILVERIO GRULLON | P. GARINO GULLOTTA | R. STUMBRIS | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D602" t="n">
+        <v>5</v>
+      </c>
+      <c r="E602" t="n">
+        <v>26</v>
+      </c>
+      <c r="F602" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G602" t="n">
+        <v>0</v>
+      </c>
+      <c r="H602" t="n">
+        <v>2</v>
+      </c>
+      <c r="I602" t="n">
+        <v>1</v>
+      </c>
+      <c r="J602" t="n">
+        <v>1</v>
+      </c>
+      <c r="K602" t="n">
+        <v>0</v>
+      </c>
+      <c r="L602" t="n">
+        <v>200</v>
+      </c>
+      <c r="M602" t="n">
+        <v>-200</v>
+      </c>
+      <c r="N602" t="n">
+        <v>1</v>
+      </c>
+      <c r="O602" t="n">
+        <v>0</v>
+      </c>
+      <c r="P602" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q602" t="n">
+        <v>0</v>
+      </c>
+      <c r="R602" t="n">
+        <v>2</v>
+      </c>
+      <c r="S602" t="n">
+        <v>0</v>
+      </c>
+      <c r="T602" t="n">
+        <v>0</v>
+      </c>
+      <c r="U602" t="n">
+        <v>1</v>
+      </c>
+      <c r="V602" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W602" t="n">
+        <v>28</v>
+      </c>
+      <c r="X602" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>A. FAURE RIBES | D. DUSCAK | G. PARHAM II | J. ARIAS GONZALEZ | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D603" t="n">
+        <v>5</v>
+      </c>
+      <c r="E603" t="n">
+        <v>82</v>
+      </c>
+      <c r="F603" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="G603" t="n">
+        <v>0</v>
+      </c>
+      <c r="H603" t="n">
+        <v>2</v>
+      </c>
+      <c r="I603" t="n">
+        <v>1</v>
+      </c>
+      <c r="J603" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="K603" t="n">
+        <v>0</v>
+      </c>
+      <c r="L603" t="n">
+        <v>106.38</v>
+      </c>
+      <c r="M603" t="n">
+        <v>-106.38</v>
+      </c>
+      <c r="N603" t="n">
+        <v>2</v>
+      </c>
+      <c r="O603" t="n">
+        <v>0</v>
+      </c>
+      <c r="P603" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q603" t="n">
+        <v>1</v>
+      </c>
+      <c r="R603" t="n">
+        <v>2</v>
+      </c>
+      <c r="S603" t="n">
+        <v>2</v>
+      </c>
+      <c r="T603" t="n">
+        <v>0</v>
+      </c>
+      <c r="U603" t="n">
+        <v>1</v>
+      </c>
+      <c r="V603" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W603" t="n">
+        <v>28</v>
+      </c>
+      <c r="X603" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>A. FAURE RIBES | D. DUSCAK | G. PARHAM II | M. TOWNES VILLAR | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D604" t="n">
+        <v>5</v>
+      </c>
+      <c r="E604" t="n">
+        <v>44</v>
+      </c>
+      <c r="F604" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G604" t="n">
+        <v>2</v>
+      </c>
+      <c r="H604" t="n">
+        <v>4</v>
+      </c>
+      <c r="I604" t="n">
+        <v>2</v>
+      </c>
+      <c r="J604" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="K604" t="n">
+        <v>100</v>
+      </c>
+      <c r="L604" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="M604" t="n">
+        <v>-112.77</v>
+      </c>
+      <c r="N604" t="n">
+        <v>2</v>
+      </c>
+      <c r="O604" t="n">
+        <v>0</v>
+      </c>
+      <c r="P604" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q604" t="n">
+        <v>0</v>
+      </c>
+      <c r="R604" t="n">
+        <v>1</v>
+      </c>
+      <c r="S604" t="n">
+        <v>2</v>
+      </c>
+      <c r="T604" t="n">
+        <v>0</v>
+      </c>
+      <c r="U604" t="n">
+        <v>0</v>
+      </c>
+      <c r="V604" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W604" t="n">
+        <v>28</v>
+      </c>
+      <c r="X604" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>D. DUSCAK | G. PARHAM II | M. TOWNES VILLAR | R. COSIALLS BORRAS | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D605" t="n">
+        <v>5</v>
+      </c>
+      <c r="E605" t="n">
+        <v>90</v>
+      </c>
+      <c r="F605" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G605" t="n">
+        <v>2</v>
+      </c>
+      <c r="H605" t="n">
+        <v>4</v>
+      </c>
+      <c r="I605" t="n">
+        <v>3</v>
+      </c>
+      <c r="J605" t="n">
+        <v>2</v>
+      </c>
+      <c r="K605" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="L605" t="n">
+        <v>200</v>
+      </c>
+      <c r="M605" t="n">
+        <v>-133.33</v>
+      </c>
+      <c r="N605" t="n">
+        <v>3</v>
+      </c>
+      <c r="O605" t="n">
+        <v>0</v>
+      </c>
+      <c r="P605" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q605" t="n">
+        <v>0</v>
+      </c>
+      <c r="R605" t="n">
+        <v>2</v>
+      </c>
+      <c r="S605" t="n">
+        <v>0</v>
+      </c>
+      <c r="T605" t="n">
+        <v>0</v>
+      </c>
+      <c r="U605" t="n">
+        <v>0</v>
+      </c>
+      <c r="V605" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W605" t="n">
+        <v>28</v>
+      </c>
+      <c r="X605" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>F. NWAOKORIE | J. ARIAS GONZALEZ | M. TOWNES VILLAR | R. COSIALLS BORRAS | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D606" t="n">
+        <v>5</v>
+      </c>
+      <c r="E606" t="n">
+        <v>10</v>
+      </c>
+      <c r="F606" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G606" t="n">
+        <v>2</v>
+      </c>
+      <c r="H606" t="n">
+        <v>0</v>
+      </c>
+      <c r="I606" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="J606" t="n">
+        <v>1</v>
+      </c>
+      <c r="K606" t="n">
+        <v>0</v>
+      </c>
+      <c r="L606" t="n">
+        <v>0</v>
+      </c>
+      <c r="M606" t="n">
+        <v>0</v>
+      </c>
+      <c r="N606" t="n">
+        <v>0</v>
+      </c>
+      <c r="O606" t="n">
+        <v>2</v>
+      </c>
+      <c r="P606" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q606" t="n">
+        <v>1</v>
+      </c>
+      <c r="R606" t="n">
+        <v>1</v>
+      </c>
+      <c r="S606" t="n">
+        <v>0</v>
+      </c>
+      <c r="T606" t="n">
+        <v>0</v>
+      </c>
+      <c r="U606" t="n">
+        <v>0</v>
+      </c>
+      <c r="V606" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W606" t="n">
+        <v>28</v>
+      </c>
+      <c r="X606" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>A. JORDA RODRIGUEZ | D. GEU | J. BONE | K. LARSEN | M. TORRES CUEVAS</t>
+        </is>
+      </c>
+      <c r="D607" t="n">
+        <v>5</v>
+      </c>
+      <c r="E607" t="n">
+        <v>206</v>
+      </c>
+      <c r="F607" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="G607" t="n">
+        <v>10</v>
+      </c>
+      <c r="H607" t="n">
+        <v>4</v>
+      </c>
+      <c r="I607" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="J607" t="n">
+        <v>6</v>
+      </c>
+      <c r="K607" t="n">
+        <v>173.61</v>
+      </c>
+      <c r="L607" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="M607" t="n">
+        <v>106.94</v>
+      </c>
+      <c r="N607" t="n">
+        <v>5</v>
+      </c>
+      <c r="O607" t="n">
+        <v>4</v>
+      </c>
+      <c r="P607" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q607" t="n">
+        <v>1</v>
+      </c>
+      <c r="R607" t="n">
+        <v>7</v>
+      </c>
+      <c r="S607" t="n">
+        <v>0</v>
+      </c>
+      <c r="T607" t="n">
+        <v>0</v>
+      </c>
+      <c r="U607" t="n">
+        <v>1</v>
+      </c>
+      <c r="V607" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W607" t="n">
+        <v>28</v>
+      </c>
+      <c r="X607" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>A. JORDA RODRIGUEZ | D. GEU | J. BONE | M. TORRES CUEVAS | U. MENDICOTE RUBIO</t>
+        </is>
+      </c>
+      <c r="D608" t="n">
+        <v>5</v>
+      </c>
+      <c r="E608" t="n">
+        <v>10</v>
+      </c>
+      <c r="F608" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G608" t="n">
+        <v>0</v>
+      </c>
+      <c r="H608" t="n">
+        <v>0</v>
+      </c>
+      <c r="I608" t="n">
+        <v>0</v>
+      </c>
+      <c r="J608" t="n">
+        <v>0</v>
+      </c>
+      <c r="K608" t="n">
+        <v>0</v>
+      </c>
+      <c r="L608" t="n">
+        <v>0</v>
+      </c>
+      <c r="M608" t="n">
+        <v>0</v>
+      </c>
+      <c r="N608" t="n">
+        <v>0</v>
+      </c>
+      <c r="O608" t="n">
+        <v>0</v>
+      </c>
+      <c r="P608" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q608" t="n">
+        <v>0</v>
+      </c>
+      <c r="R608" t="n">
+        <v>0</v>
+      </c>
+      <c r="S608" t="n">
+        <v>0</v>
+      </c>
+      <c r="T608" t="n">
+        <v>0</v>
+      </c>
+      <c r="U608" t="n">
+        <v>0</v>
+      </c>
+      <c r="V608" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W608" t="n">
+        <v>28</v>
+      </c>
+      <c r="X608" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2486505</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>A. JORDA RODRIGUEZ | J. BONE | J. MWEMA | K. LARSEN | M. TORRES CUEVAS</t>
+        </is>
+      </c>
+      <c r="D609" t="n">
+        <v>5</v>
+      </c>
+      <c r="E609" t="n">
+        <v>10</v>
+      </c>
+      <c r="F609" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G609" t="n">
+        <v>0</v>
+      </c>
+      <c r="H609" t="n">
+        <v>2</v>
+      </c>
+      <c r="I609" t="n">
+        <v>1</v>
+      </c>
+      <c r="J609" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="K609" t="n">
+        <v>0</v>
+      </c>
+      <c r="L609" t="n">
+        <v>0</v>
+      </c>
+      <c r="M609" t="n">
+        <v>0</v>
+      </c>
+      <c r="N609" t="n">
+        <v>1</v>
+      </c>
+      <c r="O609" t="n">
+        <v>0</v>
+      </c>
+      <c r="P609" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q609" t="n">
+        <v>0</v>
+      </c>
+      <c r="R609" t="n">
+        <v>0</v>
+      </c>
+      <c r="S609" t="n">
+        <v>2</v>
+      </c>
+      <c r="T609" t="n">
+        <v>0</v>
+      </c>
+      <c r="U609" t="n">
+        <v>1</v>
+      </c>
+      <c r="V609" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W609" t="n">
+        <v>28</v>
+      </c>
+      <c r="X609" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2486513</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>C. DE SOUZA PACHECO | I. DIOP GAYE | J. CREMO | P. JORGENSEN | S. BARRO</t>
+        </is>
+      </c>
+      <c r="D610" t="n">
+        <v>5</v>
+      </c>
+      <c r="E610" t="n">
+        <v>47</v>
+      </c>
+      <c r="F610" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G610" t="n">
+        <v>0</v>
+      </c>
+      <c r="H610" t="n">
+        <v>4</v>
+      </c>
+      <c r="I610" t="n">
+        <v>2</v>
+      </c>
+      <c r="J610" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="K610" t="n">
+        <v>0</v>
+      </c>
+      <c r="L610" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="M610" t="n">
+        <v>-212.77</v>
+      </c>
+      <c r="N610" t="n">
+        <v>2</v>
+      </c>
+      <c r="O610" t="n">
+        <v>0</v>
+      </c>
+      <c r="P610" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q610" t="n">
+        <v>0</v>
+      </c>
+      <c r="R610" t="n">
+        <v>1</v>
+      </c>
+      <c r="S610" t="n">
+        <v>2</v>
+      </c>
+      <c r="T610" t="n">
+        <v>0</v>
+      </c>
+      <c r="U610" t="n">
+        <v>0</v>
+      </c>
+      <c r="V610" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W610" t="n">
+        <v>29</v>
+      </c>
+      <c r="X610" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO vs LEYMA CORUÑA</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2486513</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>C. DE SOUZA PACHECO | I. DIOP GAYE | J. DIAZ ALEJANO | P. JORGENSEN | S. BARRO</t>
+        </is>
+      </c>
+      <c r="D611" t="n">
+        <v>5</v>
+      </c>
+      <c r="E611" t="n">
+        <v>37</v>
+      </c>
+      <c r="F611" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G611" t="n">
+        <v>0</v>
+      </c>
+      <c r="H611" t="n">
+        <v>3</v>
+      </c>
+      <c r="I611" t="n">
+        <v>1</v>
+      </c>
+      <c r="J611" t="n">
+        <v>2</v>
+      </c>
+      <c r="K611" t="n">
+        <v>0</v>
+      </c>
+      <c r="L611" t="n">
+        <v>150</v>
+      </c>
+      <c r="M611" t="n">
+        <v>-150</v>
+      </c>
+      <c r="N611" t="n">
+        <v>0</v>
+      </c>
+      <c r="O611" t="n">
+        <v>0</v>
+      </c>
+      <c r="P611" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q611" t="n">
+        <v>0</v>
+      </c>
+      <c r="R611" t="n">
+        <v>2</v>
+      </c>
+      <c r="S611" t="n">
+        <v>0</v>
+      </c>
+      <c r="T611" t="n">
+        <v>0</v>
+      </c>
+      <c r="U611" t="n">
+        <v>0</v>
+      </c>
+      <c r="V611" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W611" t="n">
+        <v>29</v>
+      </c>
+      <c r="X611" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO vs LEYMA CORUÑA</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2486513</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>A. GALAN POZO | D. DE SOUSA ANJO BRITO | D. KRAVIC | L. WESTERMANN | T. MUNNINGS</t>
+        </is>
+      </c>
+      <c r="D612" t="n">
+        <v>5</v>
+      </c>
+      <c r="E612" t="n">
+        <v>37</v>
+      </c>
+      <c r="F612" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G612" t="n">
+        <v>3</v>
+      </c>
+      <c r="H612" t="n">
+        <v>0</v>
+      </c>
+      <c r="I612" t="n">
+        <v>2</v>
+      </c>
+      <c r="J612" t="n">
+        <v>1</v>
+      </c>
+      <c r="K612" t="n">
+        <v>150</v>
+      </c>
+      <c r="L612" t="n">
+        <v>0</v>
+      </c>
+      <c r="M612" t="n">
+        <v>150</v>
+      </c>
+      <c r="N612" t="n">
+        <v>2</v>
+      </c>
+      <c r="O612" t="n">
+        <v>0</v>
+      </c>
+      <c r="P612" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q612" t="n">
+        <v>0</v>
+      </c>
+      <c r="R612" t="n">
+        <v>0</v>
+      </c>
+      <c r="S612" t="n">
+        <v>0</v>
+      </c>
+      <c r="T612" t="n">
+        <v>1</v>
+      </c>
+      <c r="U612" t="n">
+        <v>0</v>
+      </c>
+      <c r="V612" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W612" t="n">
+        <v>29</v>
+      </c>
+      <c r="X612" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO vs LEYMA CORUÑA</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2486513</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>D. DE SOUSA ANJO BRITO | D. KRAVIC | S. QUINTELA SALVADOR | T. MUNNINGS</t>
+        </is>
+      </c>
+      <c r="D613" t="n">
+        <v>4</v>
+      </c>
+      <c r="E613" t="n">
+        <v>47</v>
+      </c>
+      <c r="F613" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G613" t="n">
+        <v>4</v>
+      </c>
+      <c r="H613" t="n">
+        <v>0</v>
+      </c>
+      <c r="I613" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J613" t="n">
+        <v>2</v>
+      </c>
+      <c r="K613" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="L613" t="n">
+        <v>0</v>
+      </c>
+      <c r="M613" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="N613" t="n">
+        <v>1</v>
+      </c>
+      <c r="O613" t="n">
+        <v>2</v>
+      </c>
+      <c r="P613" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q613" t="n">
+        <v>0</v>
+      </c>
+      <c r="R613" t="n">
+        <v>2</v>
+      </c>
+      <c r="S613" t="n">
+        <v>0</v>
+      </c>
+      <c r="T613" t="n">
+        <v>0</v>
+      </c>
+      <c r="U613" t="n">
+        <v>0</v>
+      </c>
+      <c r="V613" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W613" t="n">
+        <v>29</v>
+      </c>
+      <c r="X613" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO vs LEYMA CORUÑA</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2486515</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>A. VRABAC | G. KALSCHEUR | I. VAZQUEZ PEREZ | R. DIAS MARQUES LISBOA SANTOS | R. GILL</t>
+        </is>
+      </c>
+      <c r="D614" t="n">
+        <v>5</v>
+      </c>
+      <c r="E614" t="n">
+        <v>22</v>
+      </c>
+      <c r="F614" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G614" t="n">
+        <v>0</v>
+      </c>
+      <c r="H614" t="n">
+        <v>1</v>
+      </c>
+      <c r="I614" t="n">
+        <v>0</v>
+      </c>
+      <c r="J614" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K614" t="n">
+        <v>0</v>
+      </c>
+      <c r="L614" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="M614" t="n">
+        <v>0</v>
+      </c>
+      <c r="N614" t="n">
+        <v>1</v>
+      </c>
+      <c r="O614" t="n">
+        <v>0</v>
+      </c>
+      <c r="P614" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q614" t="n">
+        <v>1</v>
+      </c>
+      <c r="R614" t="n">
+        <v>0</v>
+      </c>
+      <c r="S614" t="n">
+        <v>2</v>
+      </c>
+      <c r="T614" t="n">
+        <v>0</v>
+      </c>
+      <c r="U614" t="n">
+        <v>0</v>
+      </c>
+      <c r="V614" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W614" t="n">
+        <v>29</v>
+      </c>
+      <c r="X614" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA vs CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2486515</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>A. VRABAC | G. KALSCHEUR | R. DIAS MARQUES LISBOA SANTOS | R. GILL | S. MC DONNELL</t>
+        </is>
+      </c>
+      <c r="D615" t="n">
+        <v>5</v>
+      </c>
+      <c r="E615" t="n">
+        <v>64</v>
+      </c>
+      <c r="F615" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G615" t="n">
+        <v>4</v>
+      </c>
+      <c r="H615" t="n">
+        <v>8</v>
+      </c>
+      <c r="I615" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="J615" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="K615" t="n">
+        <v>106.38</v>
+      </c>
+      <c r="L615" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="M615" t="n">
+        <v>-106.38</v>
+      </c>
+      <c r="N615" t="n">
+        <v>2</v>
+      </c>
+      <c r="O615" t="n">
+        <v>4</v>
+      </c>
+      <c r="P615" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q615" t="n">
+        <v>0</v>
+      </c>
+      <c r="R615" t="n">
+        <v>2</v>
+      </c>
+      <c r="S615" t="n">
+        <v>4</v>
+      </c>
+      <c r="T615" t="n">
+        <v>0</v>
+      </c>
+      <c r="U615" t="n">
+        <v>0</v>
+      </c>
+      <c r="V615" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W615" t="n">
+        <v>29</v>
+      </c>
+      <c r="X615" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA vs CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2486515</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>D. ALDERETE DIAZ | D. LOVE | J. YU | M. LAPORNIK | P. HERNANDEZ MONTENEGRO</t>
+        </is>
+      </c>
+      <c r="D616" t="n">
+        <v>5</v>
+      </c>
+      <c r="E616" t="n">
+        <v>52</v>
+      </c>
+      <c r="F616" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G616" t="n">
+        <v>1</v>
+      </c>
+      <c r="H616" t="n">
+        <v>4</v>
+      </c>
+      <c r="I616" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J616" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="K616" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="L616" t="n">
+        <v>138.89</v>
+      </c>
+      <c r="M616" t="n">
+        <v>-25.25</v>
+      </c>
+      <c r="N616" t="n">
+        <v>0</v>
+      </c>
+      <c r="O616" t="n">
+        <v>2</v>
+      </c>
+      <c r="P616" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q616" t="n">
+        <v>0</v>
+      </c>
+      <c r="R616" t="n">
+        <v>3</v>
+      </c>
+      <c r="S616" t="n">
+        <v>2</v>
+      </c>
+      <c r="T616" t="n">
+        <v>0</v>
+      </c>
+      <c r="U616" t="n">
+        <v>1</v>
+      </c>
+      <c r="V616" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W616" t="n">
+        <v>29</v>
+      </c>
+      <c r="X616" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA vs CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2486515</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>D. ALDERETE DIAZ | D. VAN OOSTRUM | J. YU | M. LAPORNIK | P. HERNANDEZ MONTENEGRO</t>
+        </is>
+      </c>
+      <c r="D617" t="n">
+        <v>5</v>
+      </c>
+      <c r="E617" t="n">
+        <v>23</v>
+      </c>
+      <c r="F617" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G617" t="n">
+        <v>4</v>
+      </c>
+      <c r="H617" t="n">
+        <v>0</v>
+      </c>
+      <c r="I617" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J617" t="n">
+        <v>0</v>
+      </c>
+      <c r="K617" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="L617" t="n">
+        <v>0</v>
+      </c>
+      <c r="M617" t="n">
+        <v>0</v>
+      </c>
+      <c r="N617" t="n">
+        <v>1</v>
+      </c>
+      <c r="O617" t="n">
+        <v>2</v>
+      </c>
+      <c r="P617" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q617" t="n">
+        <v>0</v>
+      </c>
+      <c r="R617" t="n">
+        <v>0</v>
+      </c>
+      <c r="S617" t="n">
+        <v>0</v>
+      </c>
+      <c r="T617" t="n">
+        <v>0</v>
+      </c>
+      <c r="U617" t="n">
+        <v>0</v>
+      </c>
+      <c r="V617" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W617" t="n">
+        <v>29</v>
+      </c>
+      <c r="X617" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA vs CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2486515</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>J. YU | M. LAPORNIK | P. HERNANDEZ MONTENEGRO | R. JOHNSON JR</t>
+        </is>
+      </c>
+      <c r="D618" t="n">
+        <v>4</v>
+      </c>
+      <c r="E618" t="n">
+        <v>11</v>
+      </c>
+      <c r="F618" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G618" t="n">
+        <v>4</v>
+      </c>
+      <c r="H618" t="n">
+        <v>0</v>
+      </c>
+      <c r="I618" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J618" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K618" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="L618" t="n">
+        <v>0</v>
+      </c>
+      <c r="M618" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="N618" t="n">
+        <v>1</v>
+      </c>
+      <c r="O618" t="n">
+        <v>2</v>
+      </c>
+      <c r="P618" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q618" t="n">
+        <v>0</v>
+      </c>
+      <c r="R618" t="n">
+        <v>0</v>
+      </c>
+      <c r="S618" t="n">
+        <v>2</v>
+      </c>
+      <c r="T618" t="n">
+        <v>0</v>
+      </c>
+      <c r="U618" t="n">
+        <v>0</v>
+      </c>
+      <c r="V618" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W618" t="n">
+        <v>29</v>
+      </c>
+      <c r="X618" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA vs CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2486516</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>D. DUSCAK | G. PARHAM II | M. TOWNES VILLAR | R. COSIALLS BORRAS | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D619" t="n">
+        <v>5</v>
+      </c>
+      <c r="E619" t="n">
+        <v>71</v>
+      </c>
+      <c r="F619" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G619" t="n">
+        <v>0</v>
+      </c>
+      <c r="H619" t="n">
+        <v>3</v>
+      </c>
+      <c r="I619" t="n">
+        <v>1</v>
+      </c>
+      <c r="J619" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="K619" t="n">
+        <v>0</v>
+      </c>
+      <c r="L619" t="n">
+        <v>208.33</v>
+      </c>
+      <c r="M619" t="n">
+        <v>-208.33</v>
+      </c>
+      <c r="N619" t="n">
+        <v>1</v>
+      </c>
+      <c r="O619" t="n">
+        <v>0</v>
+      </c>
+      <c r="P619" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q619" t="n">
+        <v>0</v>
+      </c>
+      <c r="R619" t="n">
+        <v>2</v>
+      </c>
+      <c r="S619" t="n">
+        <v>1</v>
+      </c>
+      <c r="T619" t="n">
+        <v>1</v>
+      </c>
+      <c r="U619" t="n">
+        <v>2</v>
+      </c>
+      <c r="V619" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W619" t="n">
+        <v>29</v>
+      </c>
+      <c r="X619" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2486516</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>B. DE BISSCHOP | D. MANCHON CRESPO | J. BELEMENE-DZABATOU | M. DIAZ | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D620" t="n">
+        <v>5</v>
+      </c>
+      <c r="E620" t="n">
+        <v>41</v>
+      </c>
+      <c r="F620" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G620" t="n">
+        <v>3</v>
+      </c>
+      <c r="H620" t="n">
+        <v>0</v>
+      </c>
+      <c r="I620" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J620" t="n">
+        <v>1</v>
+      </c>
+      <c r="K620" t="n">
+        <v>208.33</v>
+      </c>
+      <c r="L620" t="n">
+        <v>0</v>
+      </c>
+      <c r="M620" t="n">
+        <v>208.33</v>
+      </c>
+      <c r="N620" t="n">
+        <v>2</v>
+      </c>
+      <c r="O620" t="n">
+        <v>1</v>
+      </c>
+      <c r="P620" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q620" t="n">
+        <v>2</v>
+      </c>
+      <c r="R620" t="n">
+        <v>1</v>
+      </c>
+      <c r="S620" t="n">
+        <v>0</v>
+      </c>
+      <c r="T620" t="n">
+        <v>0</v>
+      </c>
+      <c r="U620" t="n">
+        <v>0</v>
+      </c>
+      <c r="V620" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W620" t="n">
+        <v>29</v>
+      </c>
+      <c r="X620" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2486516</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>B. DE BISSCHOP | J. BELEMENE-DZABATOU | M. DIAZ | P. ALI | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D621" t="n">
+        <v>5</v>
+      </c>
+      <c r="E621" t="n">
+        <v>30</v>
+      </c>
+      <c r="F621" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G621" t="n">
+        <v>0</v>
+      </c>
+      <c r="H621" t="n">
+        <v>0</v>
+      </c>
+      <c r="I621" t="n">
+        <v>0</v>
+      </c>
+      <c r="J621" t="n">
+        <v>0</v>
+      </c>
+      <c r="K621" t="n">
+        <v>0</v>
+      </c>
+      <c r="L621" t="n">
+        <v>0</v>
+      </c>
+      <c r="M621" t="n">
+        <v>0</v>
+      </c>
+      <c r="N621" t="n">
+        <v>0</v>
+      </c>
+      <c r="O621" t="n">
+        <v>0</v>
+      </c>
+      <c r="P621" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q621" t="n">
+        <v>0</v>
+      </c>
+      <c r="R621" t="n">
+        <v>0</v>
+      </c>
+      <c r="S621" t="n">
+        <v>0</v>
+      </c>
+      <c r="T621" t="n">
+        <v>0</v>
+      </c>
+      <c r="U621" t="n">
+        <v>0</v>
+      </c>
+      <c r="V621" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W621" t="n">
+        <v>29</v>
+      </c>
+      <c r="X621" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA vs ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | B. PREPELIC | J. ROUND | J. VAN ZEGEREN | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D622" t="n">
+        <v>5</v>
+      </c>
+      <c r="E622" t="n">
+        <v>51</v>
+      </c>
+      <c r="F622" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G622" t="n">
+        <v>2</v>
+      </c>
+      <c r="H622" t="n">
+        <v>0</v>
+      </c>
+      <c r="I622" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="J622" t="n">
+        <v>2</v>
+      </c>
+      <c r="K622" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="L622" t="n">
+        <v>0</v>
+      </c>
+      <c r="M622" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="N622" t="n">
+        <v>0</v>
+      </c>
+      <c r="O622" t="n">
+        <v>2</v>
+      </c>
+      <c r="P622" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q622" t="n">
+        <v>0</v>
+      </c>
+      <c r="R622" t="n">
+        <v>0</v>
+      </c>
+      <c r="S622" t="n">
+        <v>0</v>
+      </c>
+      <c r="T622" t="n">
+        <v>2</v>
+      </c>
+      <c r="U622" t="n">
+        <v>0</v>
+      </c>
+      <c r="V622" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W622" t="n">
+        <v>29</v>
+      </c>
+      <c r="X622" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | B. PREPELIC | J. ROUND | O. LO | T. NASPLER PERAIRE</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>5</v>
+      </c>
+      <c r="E623" t="n">
+        <v>11</v>
+      </c>
+      <c r="F623" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G623" t="n">
+        <v>2</v>
+      </c>
+      <c r="H623" t="n">
+        <v>0</v>
+      </c>
+      <c r="I623" t="n">
+        <v>1</v>
+      </c>
+      <c r="J623" t="n">
+        <v>1</v>
+      </c>
+      <c r="K623" t="n">
+        <v>200</v>
+      </c>
+      <c r="L623" t="n">
+        <v>0</v>
+      </c>
+      <c r="M623" t="n">
+        <v>200</v>
+      </c>
+      <c r="N623" t="n">
+        <v>1</v>
+      </c>
+      <c r="O623" t="n">
+        <v>0</v>
+      </c>
+      <c r="P623" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q623" t="n">
+        <v>0</v>
+      </c>
+      <c r="R623" t="n">
+        <v>1</v>
+      </c>
+      <c r="S623" t="n">
+        <v>0</v>
+      </c>
+      <c r="T623" t="n">
+        <v>0</v>
+      </c>
+      <c r="U623" t="n">
+        <v>0</v>
+      </c>
+      <c r="V623" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W623" t="n">
+        <v>29</v>
+      </c>
+      <c r="X623" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | B. PREPELIC | J. VAN ZEGEREN | T. NASPLER PERAIRE | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>5</v>
+      </c>
+      <c r="E624" t="n">
+        <v>35</v>
+      </c>
+      <c r="F624" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G624" t="n">
+        <v>0</v>
+      </c>
+      <c r="H624" t="n">
+        <v>2</v>
+      </c>
+      <c r="I624" t="n">
+        <v>1</v>
+      </c>
+      <c r="J624" t="n">
+        <v>1</v>
+      </c>
+      <c r="K624" t="n">
+        <v>0</v>
+      </c>
+      <c r="L624" t="n">
+        <v>200</v>
+      </c>
+      <c r="M624" t="n">
+        <v>-200</v>
+      </c>
+      <c r="N624" t="n">
+        <v>0</v>
+      </c>
+      <c r="O624" t="n">
+        <v>0</v>
+      </c>
+      <c r="P624" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q624" t="n">
+        <v>0</v>
+      </c>
+      <c r="R624" t="n">
+        <v>1</v>
+      </c>
+      <c r="S624" t="n">
+        <v>0</v>
+      </c>
+      <c r="T624" t="n">
+        <v>0</v>
+      </c>
+      <c r="U624" t="n">
+        <v>0</v>
+      </c>
+      <c r="V624" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W624" t="n">
+        <v>29</v>
+      </c>
+      <c r="X624" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>B. PREPELIC | C. ROGERS | J. PERIS CRESPO | J. VAN ZEGEREN | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>5</v>
+      </c>
+      <c r="E625" t="n">
+        <v>16</v>
+      </c>
+      <c r="F625" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G625" t="n">
+        <v>0</v>
+      </c>
+      <c r="H625" t="n">
+        <v>2</v>
+      </c>
+      <c r="I625" t="n">
+        <v>0</v>
+      </c>
+      <c r="J625" t="n">
+        <v>1</v>
+      </c>
+      <c r="K625" t="n">
+        <v>0</v>
+      </c>
+      <c r="L625" t="n">
+        <v>200</v>
+      </c>
+      <c r="M625" t="n">
+        <v>0</v>
+      </c>
+      <c r="N625" t="n">
+        <v>0</v>
+      </c>
+      <c r="O625" t="n">
+        <v>0</v>
+      </c>
+      <c r="P625" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q625" t="n">
+        <v>0</v>
+      </c>
+      <c r="R625" t="n">
+        <v>1</v>
+      </c>
+      <c r="S625" t="n">
+        <v>0</v>
+      </c>
+      <c r="T625" t="n">
+        <v>0</v>
+      </c>
+      <c r="U625" t="n">
+        <v>0</v>
+      </c>
+      <c r="V625" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W625" t="n">
+        <v>29</v>
+      </c>
+      <c r="X625" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>B. PREPELIC | C. ROGERS | J. VAN ZEGEREN | T. NASPLER PERAIRE | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>5</v>
+      </c>
+      <c r="E626" t="n">
+        <v>80</v>
+      </c>
+      <c r="F626" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G626" t="n">
+        <v>1</v>
+      </c>
+      <c r="H626" t="n">
+        <v>0</v>
+      </c>
+      <c r="I626" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J626" t="n">
+        <v>3</v>
+      </c>
+      <c r="K626" t="n">
+        <v>53.19</v>
+      </c>
+      <c r="L626" t="n">
+        <v>0</v>
+      </c>
+      <c r="M626" t="n">
+        <v>53.19</v>
+      </c>
+      <c r="N626" t="n">
+        <v>2</v>
+      </c>
+      <c r="O626" t="n">
+        <v>2</v>
+      </c>
+      <c r="P626" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q626" t="n">
+        <v>1</v>
+      </c>
+      <c r="R626" t="n">
+        <v>3</v>
+      </c>
+      <c r="S626" t="n">
+        <v>0</v>
+      </c>
+      <c r="T626" t="n">
+        <v>1</v>
+      </c>
+      <c r="U626" t="n">
+        <v>1</v>
+      </c>
+      <c r="V626" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W626" t="n">
+        <v>29</v>
+      </c>
+      <c r="X626" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>C. ROGERS | D. KRISTENSEN | J. PERIS CRESPO | J. ROUND | O. LO</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>5</v>
+      </c>
+      <c r="E627" t="n">
+        <v>100</v>
+      </c>
+      <c r="F627" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="G627" t="n">
+        <v>2</v>
+      </c>
+      <c r="H627" t="n">
+        <v>3</v>
+      </c>
+      <c r="I627" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J627" t="n">
+        <v>2</v>
+      </c>
+      <c r="K627" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="L627" t="n">
+        <v>150</v>
+      </c>
+      <c r="M627" t="n">
+        <v>77.27</v>
+      </c>
+      <c r="N627" t="n">
+        <v>1</v>
+      </c>
+      <c r="O627" t="n">
+        <v>2</v>
+      </c>
+      <c r="P627" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q627" t="n">
+        <v>2</v>
+      </c>
+      <c r="R627" t="n">
+        <v>3</v>
+      </c>
+      <c r="S627" t="n">
+        <v>0</v>
+      </c>
+      <c r="T627" t="n">
+        <v>0</v>
+      </c>
+      <c r="U627" t="n">
+        <v>1</v>
+      </c>
+      <c r="V627" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W627" t="n">
+        <v>29</v>
+      </c>
+      <c r="X627" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>A. SCARIOLO ARES | B. VAZQUEZ ARRAIZA | J. ARAMBURU LAMY | L. SMITH | O. MATULIONIS</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>5</v>
+      </c>
+      <c r="E628" t="n">
+        <v>17</v>
+      </c>
+      <c r="F628" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G628" t="n">
+        <v>3</v>
+      </c>
+      <c r="H628" t="n">
+        <v>0</v>
+      </c>
+      <c r="I628" t="n">
+        <v>1</v>
+      </c>
+      <c r="J628" t="n">
+        <v>0</v>
+      </c>
+      <c r="K628" t="n">
+        <v>300</v>
+      </c>
+      <c r="L628" t="n">
+        <v>0</v>
+      </c>
+      <c r="M628" t="n">
+        <v>0</v>
+      </c>
+      <c r="N628" t="n">
+        <v>1</v>
+      </c>
+      <c r="O628" t="n">
+        <v>0</v>
+      </c>
+      <c r="P628" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q628" t="n">
+        <v>0</v>
+      </c>
+      <c r="R628" t="n">
+        <v>0</v>
+      </c>
+      <c r="S628" t="n">
+        <v>0</v>
+      </c>
+      <c r="T628" t="n">
+        <v>0</v>
+      </c>
+      <c r="U628" t="n">
+        <v>0</v>
+      </c>
+      <c r="V628" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W628" t="n">
+        <v>29</v>
+      </c>
+      <c r="X628" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>A. SCARIOLO ARES | B. VAZQUEZ ARRAIZA | J. ARAMBURU LAMY | O. MATULIONIS | P. BOMBINO PARADA</t>
+        </is>
+      </c>
+      <c r="D629" t="n">
+        <v>5</v>
+      </c>
+      <c r="E629" t="n">
+        <v>252</v>
+      </c>
+      <c r="F629" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G629" t="n">
+        <v>2</v>
+      </c>
+      <c r="H629" t="n">
+        <v>7</v>
+      </c>
+      <c r="I629" t="n">
+        <v>8</v>
+      </c>
+      <c r="J629" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="K629" t="n">
+        <v>25</v>
+      </c>
+      <c r="L629" t="n">
+        <v>91.62</v>
+      </c>
+      <c r="M629" t="n">
+        <v>-66.62</v>
+      </c>
+      <c r="N629" t="n">
+        <v>7</v>
+      </c>
+      <c r="O629" t="n">
+        <v>0</v>
+      </c>
+      <c r="P629" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q629" t="n">
+        <v>2</v>
+      </c>
+      <c r="R629" t="n">
+        <v>4</v>
+      </c>
+      <c r="S629" t="n">
+        <v>6</v>
+      </c>
+      <c r="T629" t="n">
+        <v>4</v>
+      </c>
+      <c r="U629" t="n">
+        <v>3</v>
+      </c>
+      <c r="V629" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W629" t="n">
+        <v>29</v>
+      </c>
+      <c r="X629" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2486518</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>A. SCARIOLO ARES | J. ARAMBURU LAMY | J. BOCCA | O. MATULIONIS | P. BOMBINO PARADA</t>
+        </is>
+      </c>
+      <c r="D630" t="n">
+        <v>5</v>
+      </c>
+      <c r="E630" t="n">
+        <v>24</v>
+      </c>
+      <c r="F630" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G630" t="n">
+        <v>2</v>
+      </c>
+      <c r="H630" t="n">
+        <v>0</v>
+      </c>
+      <c r="I630" t="n">
+        <v>1</v>
+      </c>
+      <c r="J630" t="n">
+        <v>0</v>
+      </c>
+      <c r="K630" t="n">
+        <v>200</v>
+      </c>
+      <c r="L630" t="n">
+        <v>0</v>
+      </c>
+      <c r="M630" t="n">
+        <v>0</v>
+      </c>
+      <c r="N630" t="n">
+        <v>1</v>
+      </c>
+      <c r="O630" t="n">
+        <v>0</v>
+      </c>
+      <c r="P630" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q630" t="n">
+        <v>0</v>
+      </c>
+      <c r="R630" t="n">
+        <v>0</v>
+      </c>
+      <c r="S630" t="n">
+        <v>0</v>
+      </c>
+      <c r="T630" t="n">
+        <v>0</v>
+      </c>
+      <c r="U630" t="n">
+        <v>0</v>
+      </c>
+      <c r="V630" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W630" t="n">
+        <v>29</v>
+      </c>
+      <c r="X630" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA vs CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2486514</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | A. MARTIN MARIN | J. LOPEZ SANTANA | K. WEBSTER | S. SVEJCAR</t>
+        </is>
+      </c>
+      <c r="D631" t="n">
+        <v>5</v>
+      </c>
+      <c r="E631" t="n">
+        <v>5</v>
+      </c>
+      <c r="F631" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G631" t="n">
+        <v>2</v>
+      </c>
+      <c r="H631" t="n">
+        <v>0</v>
+      </c>
+      <c r="I631" t="n">
+        <v>1</v>
+      </c>
+      <c r="J631" t="n">
+        <v>0</v>
+      </c>
+      <c r="K631" t="n">
+        <v>200</v>
+      </c>
+      <c r="L631" t="n">
+        <v>0</v>
+      </c>
+      <c r="M631" t="n">
+        <v>0</v>
+      </c>
+      <c r="N631" t="n">
+        <v>1</v>
+      </c>
+      <c r="O631" t="n">
+        <v>0</v>
+      </c>
+      <c r="P631" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q631" t="n">
+        <v>0</v>
+      </c>
+      <c r="R631" t="n">
+        <v>0</v>
+      </c>
+      <c r="S631" t="n">
+        <v>0</v>
+      </c>
+      <c r="T631" t="n">
+        <v>0</v>
+      </c>
+      <c r="U631" t="n">
+        <v>0</v>
+      </c>
+      <c r="V631" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W631" t="n">
+        <v>29</v>
+      </c>
+      <c r="X631" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA vs GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2486514</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | A. MARTIN MARIN | J. LOPEZ SANTANA | K. WEBSTER | V. FAVERANI TATSCH</t>
+        </is>
+      </c>
+      <c r="D632" t="n">
+        <v>5</v>
+      </c>
+      <c r="E632" t="n">
+        <v>18</v>
+      </c>
+      <c r="F632" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G632" t="n">
+        <v>2</v>
+      </c>
+      <c r="H632" t="n">
+        <v>4</v>
+      </c>
+      <c r="I632" t="n">
+        <v>2</v>
+      </c>
+      <c r="J632" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="K632" t="n">
+        <v>100</v>
+      </c>
+      <c r="L632" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="M632" t="n">
+        <v>-127.27</v>
+      </c>
+      <c r="N632" t="n">
+        <v>2</v>
+      </c>
+      <c r="O632" t="n">
+        <v>0</v>
+      </c>
+      <c r="P632" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q632" t="n">
+        <v>0</v>
+      </c>
+      <c r="R632" t="n">
+        <v>0</v>
+      </c>
+      <c r="S632" t="n">
+        <v>4</v>
+      </c>
+      <c r="T632" t="n">
+        <v>0</v>
+      </c>
+      <c r="U632" t="n">
+        <v>0</v>
+      </c>
+      <c r="V632" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W632" t="n">
+        <v>29</v>
+      </c>
+      <c r="X632" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA vs GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2486514</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | A. MARTIN MARIN | K. WEBSTER | S. SVEJCAR | V. FAVERANI TATSCH</t>
+        </is>
+      </c>
+      <c r="D633" t="n">
+        <v>5</v>
+      </c>
+      <c r="E633" t="n">
+        <v>215</v>
+      </c>
+      <c r="F633" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="G633" t="n">
+        <v>4</v>
+      </c>
+      <c r="H633" t="n">
+        <v>8</v>
+      </c>
+      <c r="I633" t="n">
+        <v>4</v>
+      </c>
+      <c r="J633" t="n">
+        <v>5</v>
+      </c>
+      <c r="K633" t="n">
+        <v>100</v>
+      </c>
+      <c r="L633" t="n">
+        <v>160</v>
+      </c>
+      <c r="M633" t="n">
+        <v>-60</v>
+      </c>
+      <c r="N633" t="n">
+        <v>5</v>
+      </c>
+      <c r="O633" t="n">
+        <v>0</v>
+      </c>
+      <c r="P633" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q633" t="n">
+        <v>1</v>
+      </c>
+      <c r="R633" t="n">
+        <v>7</v>
+      </c>
+      <c r="S633" t="n">
+        <v>0</v>
+      </c>
+      <c r="T633" t="n">
+        <v>2</v>
+      </c>
+      <c r="U633" t="n">
+        <v>4</v>
+      </c>
+      <c r="V633" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W633" t="n">
+        <v>29</v>
+      </c>
+      <c r="X633" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA vs GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2486514</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | J. LOPEZ SANTANA | K. WEBSTER | S. SVEJCAR | V. FAVERANI TATSCH</t>
+        </is>
+      </c>
+      <c r="D634" t="n">
+        <v>5</v>
+      </c>
+      <c r="E634" t="n">
+        <v>4</v>
+      </c>
+      <c r="F634" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G634" t="n">
+        <v>0</v>
+      </c>
+      <c r="H634" t="n">
+        <v>0</v>
+      </c>
+      <c r="I634" t="n">
+        <v>0</v>
+      </c>
+      <c r="J634" t="n">
+        <v>1</v>
+      </c>
+      <c r="K634" t="n">
+        <v>0</v>
+      </c>
+      <c r="L634" t="n">
+        <v>0</v>
+      </c>
+      <c r="M634" t="n">
+        <v>0</v>
+      </c>
+      <c r="N634" t="n">
+        <v>0</v>
+      </c>
+      <c r="O634" t="n">
+        <v>0</v>
+      </c>
+      <c r="P634" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q634" t="n">
+        <v>0</v>
+      </c>
+      <c r="R634" t="n">
+        <v>0</v>
+      </c>
+      <c r="S634" t="n">
+        <v>0</v>
+      </c>
+      <c r="T634" t="n">
+        <v>1</v>
+      </c>
+      <c r="U634" t="n">
+        <v>0</v>
+      </c>
+      <c r="V634" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W634" t="n">
+        <v>29</v>
+      </c>
+      <c r="X634" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA vs GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2486514</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>A. SOLA IDDRISU | E. VICEDO AYALA | E. WEMBI | F. ZURBRIGGEN | S. LITTLESON</t>
+        </is>
+      </c>
+      <c r="D635" t="n">
+        <v>5</v>
+      </c>
+      <c r="E635" t="n">
+        <v>47</v>
+      </c>
+      <c r="F635" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G635" t="n">
+        <v>4</v>
+      </c>
+      <c r="H635" t="n">
+        <v>2</v>
+      </c>
+      <c r="I635" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="J635" t="n">
+        <v>3</v>
+      </c>
+      <c r="K635" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="L635" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="M635" t="n">
+        <v>160.61</v>
+      </c>
+      <c r="N635" t="n">
+        <v>0</v>
+      </c>
+      <c r="O635" t="n">
+        <v>4</v>
+      </c>
+      <c r="P635" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q635" t="n">
+        <v>1</v>
+      </c>
+      <c r="R635" t="n">
+        <v>3</v>
+      </c>
+      <c r="S635" t="n">
+        <v>0</v>
+      </c>
+      <c r="T635" t="n">
+        <v>0</v>
+      </c>
+      <c r="U635" t="n">
+        <v>0</v>
+      </c>
+      <c r="V635" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W635" t="n">
+        <v>29</v>
+      </c>
+      <c r="X635" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA vs GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2486514</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>A. SOLA IDDRISU | E. VICEDO AYALA | F. ZURBRIGGEN | J. LOBO MARTORELL | V. ARTEAGA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="D636" t="n">
+        <v>5</v>
+      </c>
+      <c r="E636" t="n">
+        <v>6</v>
+      </c>
+      <c r="F636" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G636" t="n">
+        <v>0</v>
+      </c>
+      <c r="H636" t="n">
+        <v>0</v>
+      </c>
+      <c r="I636" t="n">
+        <v>1</v>
+      </c>
+      <c r="J636" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K636" t="n">
+        <v>0</v>
+      </c>
+      <c r="L636" t="n">
+        <v>0</v>
+      </c>
+      <c r="M636" t="n">
+        <v>0</v>
+      </c>
+      <c r="N636" t="n">
+        <v>1</v>
+      </c>
+      <c r="O636" t="n">
+        <v>0</v>
+      </c>
+      <c r="P636" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q636" t="n">
+        <v>0</v>
+      </c>
+      <c r="R636" t="n">
+        <v>0</v>
+      </c>
+      <c r="S636" t="n">
+        <v>0</v>
+      </c>
+      <c r="T636" t="n">
+        <v>0</v>
+      </c>
+      <c r="U636" t="n">
+        <v>1</v>
+      </c>
+      <c r="V636" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W636" t="n">
+        <v>29</v>
+      </c>
+      <c r="X636" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA vs GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2486514</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>A. SOLA IDDRISU | E. VICEDO AYALA | F. ZURBRIGGEN | S. LITTLESON | V. ARTEAGA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="D637" t="n">
+        <v>5</v>
+      </c>
+      <c r="E637" t="n">
+        <v>184</v>
+      </c>
+      <c r="F637" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="G637" t="n">
+        <v>8</v>
+      </c>
+      <c r="H637" t="n">
+        <v>4</v>
+      </c>
+      <c r="I637" t="n">
+        <v>5</v>
+      </c>
+      <c r="J637" t="n">
+        <v>4</v>
+      </c>
+      <c r="K637" t="n">
+        <v>160</v>
+      </c>
+      <c r="L637" t="n">
+        <v>100</v>
+      </c>
+      <c r="M637" t="n">
+        <v>60</v>
+      </c>
+      <c r="N637" t="n">
+        <v>6</v>
+      </c>
+      <c r="O637" t="n">
+        <v>0</v>
+      </c>
+      <c r="P637" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q637" t="n">
+        <v>3</v>
+      </c>
+      <c r="R637" t="n">
+        <v>4</v>
+      </c>
+      <c r="S637" t="n">
+        <v>0</v>
+      </c>
+      <c r="T637" t="n">
+        <v>0</v>
+      </c>
+      <c r="U637" t="n">
+        <v>0</v>
+      </c>
+      <c r="V637" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W637" t="n">
+        <v>29</v>
+      </c>
+      <c r="X637" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA vs GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2486514</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>E. VICEDO AYALA | E. WEMBI | F. ZURBRIGGEN | J. LOBO MARTORELL | S. LITTLESON</t>
+        </is>
+      </c>
+      <c r="D638" t="n">
+        <v>5</v>
+      </c>
+      <c r="E638" t="n">
+        <v>5</v>
+      </c>
+      <c r="F638" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G638" t="n">
+        <v>0</v>
+      </c>
+      <c r="H638" t="n">
+        <v>2</v>
+      </c>
+      <c r="I638" t="n">
+        <v>0</v>
+      </c>
+      <c r="J638" t="n">
+        <v>1</v>
+      </c>
+      <c r="K638" t="n">
+        <v>0</v>
+      </c>
+      <c r="L638" t="n">
+        <v>200</v>
+      </c>
+      <c r="M638" t="n">
+        <v>0</v>
+      </c>
+      <c r="N638" t="n">
+        <v>0</v>
+      </c>
+      <c r="O638" t="n">
+        <v>0</v>
+      </c>
+      <c r="P638" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q638" t="n">
+        <v>0</v>
+      </c>
+      <c r="R638" t="n">
+        <v>1</v>
+      </c>
+      <c r="S638" t="n">
+        <v>0</v>
+      </c>
+      <c r="T638" t="n">
+        <v>0</v>
+      </c>
+      <c r="U638" t="n">
+        <v>0</v>
+      </c>
+      <c r="V638" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W638" t="n">
+        <v>29</v>
+      </c>
+      <c r="X638" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA vs GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2486511</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | I. CRUZ UCEDA | M. CAICEDO SANCHEZ | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D639" t="n">
+        <v>5</v>
+      </c>
+      <c r="E639" t="n">
+        <v>7</v>
+      </c>
+      <c r="F639" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G639" t="n">
+        <v>0</v>
+      </c>
+      <c r="H639" t="n">
+        <v>2</v>
+      </c>
+      <c r="I639" t="n">
+        <v>1</v>
+      </c>
+      <c r="J639" t="n">
+        <v>1</v>
+      </c>
+      <c r="K639" t="n">
+        <v>0</v>
+      </c>
+      <c r="L639" t="n">
+        <v>200</v>
+      </c>
+      <c r="M639" t="n">
+        <v>-200</v>
+      </c>
+      <c r="N639" t="n">
+        <v>0</v>
+      </c>
+      <c r="O639" t="n">
+        <v>0</v>
+      </c>
+      <c r="P639" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q639" t="n">
+        <v>0</v>
+      </c>
+      <c r="R639" t="n">
+        <v>1</v>
+      </c>
+      <c r="S639" t="n">
+        <v>0</v>
+      </c>
+      <c r="T639" t="n">
+        <v>0</v>
+      </c>
+      <c r="U639" t="n">
+        <v>0</v>
+      </c>
+      <c r="V639" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W639" t="n">
+        <v>29</v>
+      </c>
+      <c r="X639" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE vs PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2486511</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | J. GODSPOWER JOHNSON | M. CAICEDO SANCHEZ | N. HOOVER | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D640" t="n">
+        <v>5</v>
+      </c>
+      <c r="E640" t="n">
+        <v>95</v>
+      </c>
+      <c r="F640" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="G640" t="n">
+        <v>8</v>
+      </c>
+      <c r="H640" t="n">
+        <v>0</v>
+      </c>
+      <c r="I640" t="n">
+        <v>3</v>
+      </c>
+      <c r="J640" t="n">
+        <v>2</v>
+      </c>
+      <c r="K640" t="n">
+        <v>266.67</v>
+      </c>
+      <c r="L640" t="n">
+        <v>0</v>
+      </c>
+      <c r="M640" t="n">
+        <v>266.67</v>
+      </c>
+      <c r="N640" t="n">
+        <v>4</v>
+      </c>
+      <c r="O640" t="n">
+        <v>0</v>
+      </c>
+      <c r="P640" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q640" t="n">
+        <v>1</v>
+      </c>
+      <c r="R640" t="n">
+        <v>2</v>
+      </c>
+      <c r="S640" t="n">
+        <v>0</v>
+      </c>
+      <c r="T640" t="n">
+        <v>0</v>
+      </c>
+      <c r="U640" t="n">
+        <v>0</v>
+      </c>
+      <c r="V640" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W640" t="n">
+        <v>29</v>
+      </c>
+      <c r="X640" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE vs PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2486511</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | M. CAICEDO SANCHEZ | N. MC MULLEN | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>5</v>
+      </c>
+      <c r="E641" t="n">
+        <v>15</v>
+      </c>
+      <c r="F641" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G641" t="n">
+        <v>2</v>
+      </c>
+      <c r="H641" t="n">
+        <v>1</v>
+      </c>
+      <c r="I641" t="n">
+        <v>1</v>
+      </c>
+      <c r="J641" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="K641" t="n">
+        <v>200</v>
+      </c>
+      <c r="L641" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="M641" t="n">
+        <v>-27.27</v>
+      </c>
+      <c r="N641" t="n">
+        <v>1</v>
+      </c>
+      <c r="O641" t="n">
+        <v>0</v>
+      </c>
+      <c r="P641" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q641" t="n">
+        <v>0</v>
+      </c>
+      <c r="R641" t="n">
+        <v>0</v>
+      </c>
+      <c r="S641" t="n">
+        <v>1</v>
+      </c>
+      <c r="T641" t="n">
+        <v>0</v>
+      </c>
+      <c r="U641" t="n">
+        <v>0</v>
+      </c>
+      <c r="V641" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W641" t="n">
+        <v>29</v>
+      </c>
+      <c r="X641" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE vs PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2486511</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>J. GODSPOWER JOHNSON | M. CAICEDO SANCHEZ | N. HOOVER | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>5</v>
+      </c>
+      <c r="E642" t="n">
+        <v>37</v>
+      </c>
+      <c r="F642" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G642" t="n">
+        <v>0</v>
+      </c>
+      <c r="H642" t="n">
+        <v>0</v>
+      </c>
+      <c r="I642" t="n">
+        <v>0</v>
+      </c>
+      <c r="J642" t="n">
+        <v>1</v>
+      </c>
+      <c r="K642" t="n">
+        <v>0</v>
+      </c>
+      <c r="L642" t="n">
+        <v>0</v>
+      </c>
+      <c r="M642" t="n">
+        <v>0</v>
+      </c>
+      <c r="N642" t="n">
+        <v>1</v>
+      </c>
+      <c r="O642" t="n">
+        <v>0</v>
+      </c>
+      <c r="P642" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q642" t="n">
+        <v>1</v>
+      </c>
+      <c r="R642" t="n">
+        <v>1</v>
+      </c>
+      <c r="S642" t="n">
+        <v>0</v>
+      </c>
+      <c r="T642" t="n">
+        <v>0</v>
+      </c>
+      <c r="U642" t="n">
+        <v>0</v>
+      </c>
+      <c r="V642" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W642" t="n">
+        <v>29</v>
+      </c>
+      <c r="X642" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE vs PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2486511</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>A. COMENDADOR FEMENIAS | A. URDIAIN LABAYEN | G. DIKE EGUN | H. ATENCIA SUAREZ | J. FELIU ESPEJO</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>5</v>
+      </c>
+      <c r="E643" t="n">
+        <v>7</v>
+      </c>
+      <c r="F643" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G643" t="n">
+        <v>2</v>
+      </c>
+      <c r="H643" t="n">
+        <v>0</v>
+      </c>
+      <c r="I643" t="n">
+        <v>1</v>
+      </c>
+      <c r="J643" t="n">
+        <v>1</v>
+      </c>
+      <c r="K643" t="n">
+        <v>200</v>
+      </c>
+      <c r="L643" t="n">
+        <v>0</v>
+      </c>
+      <c r="M643" t="n">
+        <v>200</v>
+      </c>
+      <c r="N643" t="n">
+        <v>1</v>
+      </c>
+      <c r="O643" t="n">
+        <v>0</v>
+      </c>
+      <c r="P643" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q643" t="n">
+        <v>0</v>
+      </c>
+      <c r="R643" t="n">
+        <v>0</v>
+      </c>
+      <c r="S643" t="n">
+        <v>0</v>
+      </c>
+      <c r="T643" t="n">
+        <v>1</v>
+      </c>
+      <c r="U643" t="n">
+        <v>0</v>
+      </c>
+      <c r="V643" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W643" t="n">
+        <v>29</v>
+      </c>
+      <c r="X643" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE vs PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2486511</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>A. COMENDADOR FEMENIAS | D. SANADZE | G. DIKE EGUN | H. ATENCIA SUAREZ | J. FELIU ESPEJO</t>
+        </is>
+      </c>
+      <c r="D644" t="n">
+        <v>5</v>
+      </c>
+      <c r="E644" t="n">
+        <v>16</v>
+      </c>
+      <c r="F644" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G644" t="n">
+        <v>1</v>
+      </c>
+      <c r="H644" t="n">
+        <v>4</v>
+      </c>
+      <c r="I644" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J644" t="n">
+        <v>2</v>
+      </c>
+      <c r="K644" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="L644" t="n">
+        <v>200</v>
+      </c>
+      <c r="M644" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="N644" t="n">
+        <v>0</v>
+      </c>
+      <c r="O644" t="n">
+        <v>1</v>
+      </c>
+      <c r="P644" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q644" t="n">
+        <v>0</v>
+      </c>
+      <c r="R644" t="n">
+        <v>2</v>
+      </c>
+      <c r="S644" t="n">
+        <v>0</v>
+      </c>
+      <c r="T644" t="n">
+        <v>0</v>
+      </c>
+      <c r="U644" t="n">
+        <v>0</v>
+      </c>
+      <c r="V644" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W644" t="n">
+        <v>29</v>
+      </c>
+      <c r="X644" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE vs PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2486511</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>A. IZAW BOLAVIE | D. SANADZE | G. DIKE EGUN | H. ATENCIA SUAREZ | J. FELIU ESPEJO</t>
+        </is>
+      </c>
+      <c r="D645" t="n">
+        <v>5</v>
+      </c>
+      <c r="E645" t="n">
+        <v>131</v>
+      </c>
+      <c r="F645" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="G645" t="n">
+        <v>0</v>
+      </c>
+      <c r="H645" t="n">
+        <v>6</v>
+      </c>
+      <c r="I645" t="n">
+        <v>3</v>
+      </c>
+      <c r="J645" t="n">
+        <v>2</v>
+      </c>
+      <c r="K645" t="n">
+        <v>0</v>
+      </c>
+      <c r="L645" t="n">
+        <v>300</v>
+      </c>
+      <c r="M645" t="n">
+        <v>-300</v>
+      </c>
+      <c r="N645" t="n">
+        <v>3</v>
+      </c>
+      <c r="O645" t="n">
+        <v>0</v>
+      </c>
+      <c r="P645" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q645" t="n">
+        <v>0</v>
+      </c>
+      <c r="R645" t="n">
+        <v>4</v>
+      </c>
+      <c r="S645" t="n">
+        <v>0</v>
+      </c>
+      <c r="T645" t="n">
+        <v>0</v>
+      </c>
+      <c r="U645" t="n">
+        <v>2</v>
+      </c>
+      <c r="V645" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W645" t="n">
+        <v>29</v>
+      </c>
+      <c r="X645" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE vs PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): sync FEB data 2026-04-20 10:54
</commit_message>
<xml_diff>
--- a/data/1FEB_25_26/clutch_lineups_25_26_1FEB.xlsx
+++ b/data/1FEB_25_26/clutch_lineups_25_26_1FEB.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X645"/>
+  <dimension ref="A1:X695"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54646,6 +54646,4206 @@
         </is>
       </c>
     </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2486525</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>J. POWELL | J. YU | M. LAPORNIK | P. HERNANDEZ MONTENEGRO | R. JOHNSON JR</t>
+        </is>
+      </c>
+      <c r="D646" t="n">
+        <v>5</v>
+      </c>
+      <c r="E646" t="n">
+        <v>7</v>
+      </c>
+      <c r="F646" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G646" t="n">
+        <v>0</v>
+      </c>
+      <c r="H646" t="n">
+        <v>0</v>
+      </c>
+      <c r="I646" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J646" t="n">
+        <v>1</v>
+      </c>
+      <c r="K646" t="n">
+        <v>0</v>
+      </c>
+      <c r="L646" t="n">
+        <v>0</v>
+      </c>
+      <c r="M646" t="n">
+        <v>0</v>
+      </c>
+      <c r="N646" t="n">
+        <v>1</v>
+      </c>
+      <c r="O646" t="n">
+        <v>2</v>
+      </c>
+      <c r="P646" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q646" t="n">
+        <v>0</v>
+      </c>
+      <c r="R646" t="n">
+        <v>0</v>
+      </c>
+      <c r="S646" t="n">
+        <v>0</v>
+      </c>
+      <c r="T646" t="n">
+        <v>1</v>
+      </c>
+      <c r="U646" t="n">
+        <v>0</v>
+      </c>
+      <c r="V646" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W646" t="n">
+        <v>30</v>
+      </c>
+      <c r="X646" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2486525</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>J. MWEMA | K. LARSEN | S. HOLLANDERS | U. MENDICOTE RUBIO | Y. JOSEPH</t>
+        </is>
+      </c>
+      <c r="D647" t="n">
+        <v>5</v>
+      </c>
+      <c r="E647" t="n">
+        <v>7</v>
+      </c>
+      <c r="F647" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G647" t="n">
+        <v>0</v>
+      </c>
+      <c r="H647" t="n">
+        <v>0</v>
+      </c>
+      <c r="I647" t="n">
+        <v>1</v>
+      </c>
+      <c r="J647" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="K647" t="n">
+        <v>0</v>
+      </c>
+      <c r="L647" t="n">
+        <v>0</v>
+      </c>
+      <c r="M647" t="n">
+        <v>0</v>
+      </c>
+      <c r="N647" t="n">
+        <v>0</v>
+      </c>
+      <c r="O647" t="n">
+        <v>0</v>
+      </c>
+      <c r="P647" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q647" t="n">
+        <v>0</v>
+      </c>
+      <c r="R647" t="n">
+        <v>1</v>
+      </c>
+      <c r="S647" t="n">
+        <v>2</v>
+      </c>
+      <c r="T647" t="n">
+        <v>0</v>
+      </c>
+      <c r="U647" t="n">
+        <v>0</v>
+      </c>
+      <c r="V647" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W647" t="n">
+        <v>30</v>
+      </c>
+      <c r="X647" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE vs GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2486524</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>A. LIMA BRITO | B. DE BISSCHOP | D. MANCHON CRESPO | G. RENFROE | M. DIAZ</t>
+        </is>
+      </c>
+      <c r="D648" t="n">
+        <v>5</v>
+      </c>
+      <c r="E648" t="n">
+        <v>15</v>
+      </c>
+      <c r="F648" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G648" t="n">
+        <v>3</v>
+      </c>
+      <c r="H648" t="n">
+        <v>0</v>
+      </c>
+      <c r="I648" t="n">
+        <v>1</v>
+      </c>
+      <c r="J648" t="n">
+        <v>0</v>
+      </c>
+      <c r="K648" t="n">
+        <v>300</v>
+      </c>
+      <c r="L648" t="n">
+        <v>0</v>
+      </c>
+      <c r="M648" t="n">
+        <v>0</v>
+      </c>
+      <c r="N648" t="n">
+        <v>1</v>
+      </c>
+      <c r="O648" t="n">
+        <v>0</v>
+      </c>
+      <c r="P648" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q648" t="n">
+        <v>0</v>
+      </c>
+      <c r="R648" t="n">
+        <v>0</v>
+      </c>
+      <c r="S648" t="n">
+        <v>0</v>
+      </c>
+      <c r="T648" t="n">
+        <v>0</v>
+      </c>
+      <c r="U648" t="n">
+        <v>0</v>
+      </c>
+      <c r="V648" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W648" t="n">
+        <v>30</v>
+      </c>
+      <c r="X648" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA vs FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2486524</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>A. LIMA BRITO | B. DE BISSCHOP | G. RENFROE | M. DIAZ | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D649" t="n">
+        <v>5</v>
+      </c>
+      <c r="E649" t="n">
+        <v>4</v>
+      </c>
+      <c r="F649" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G649" t="n">
+        <v>0</v>
+      </c>
+      <c r="H649" t="n">
+        <v>0</v>
+      </c>
+      <c r="I649" t="n">
+        <v>1</v>
+      </c>
+      <c r="J649" t="n">
+        <v>0</v>
+      </c>
+      <c r="K649" t="n">
+        <v>0</v>
+      </c>
+      <c r="L649" t="n">
+        <v>0</v>
+      </c>
+      <c r="M649" t="n">
+        <v>0</v>
+      </c>
+      <c r="N649" t="n">
+        <v>0</v>
+      </c>
+      <c r="O649" t="n">
+        <v>0</v>
+      </c>
+      <c r="P649" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q649" t="n">
+        <v>0</v>
+      </c>
+      <c r="R649" t="n">
+        <v>0</v>
+      </c>
+      <c r="S649" t="n">
+        <v>0</v>
+      </c>
+      <c r="T649" t="n">
+        <v>0</v>
+      </c>
+      <c r="U649" t="n">
+        <v>0</v>
+      </c>
+      <c r="V649" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W649" t="n">
+        <v>30</v>
+      </c>
+      <c r="X649" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA vs FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2486524</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>B. DE BISSCHOP | D. MANCHON CRESPO | G. RENFROE | J. BELEMENE-DZABATOU | M. DIAZ</t>
+        </is>
+      </c>
+      <c r="D650" t="n">
+        <v>5</v>
+      </c>
+      <c r="E650" t="n">
+        <v>10</v>
+      </c>
+      <c r="F650" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G650" t="n">
+        <v>0</v>
+      </c>
+      <c r="H650" t="n">
+        <v>0</v>
+      </c>
+      <c r="I650" t="n">
+        <v>1</v>
+      </c>
+      <c r="J650" t="n">
+        <v>0</v>
+      </c>
+      <c r="K650" t="n">
+        <v>0</v>
+      </c>
+      <c r="L650" t="n">
+        <v>0</v>
+      </c>
+      <c r="M650" t="n">
+        <v>0</v>
+      </c>
+      <c r="N650" t="n">
+        <v>1</v>
+      </c>
+      <c r="O650" t="n">
+        <v>0</v>
+      </c>
+      <c r="P650" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q650" t="n">
+        <v>0</v>
+      </c>
+      <c r="R650" t="n">
+        <v>0</v>
+      </c>
+      <c r="S650" t="n">
+        <v>0</v>
+      </c>
+      <c r="T650" t="n">
+        <v>0</v>
+      </c>
+      <c r="U650" t="n">
+        <v>0</v>
+      </c>
+      <c r="V650" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W650" t="n">
+        <v>30</v>
+      </c>
+      <c r="X650" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA vs FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2486524</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>B. DE BISSCHOP | D. MANCHON CRESPO | G. RENFROE | M. DIAZ | V. ALVES BENITE</t>
+        </is>
+      </c>
+      <c r="D651" t="n">
+        <v>5</v>
+      </c>
+      <c r="E651" t="n">
+        <v>22</v>
+      </c>
+      <c r="F651" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G651" t="n">
+        <v>0</v>
+      </c>
+      <c r="H651" t="n">
+        <v>2</v>
+      </c>
+      <c r="I651" t="n">
+        <v>0</v>
+      </c>
+      <c r="J651" t="n">
+        <v>1</v>
+      </c>
+      <c r="K651" t="n">
+        <v>0</v>
+      </c>
+      <c r="L651" t="n">
+        <v>200</v>
+      </c>
+      <c r="M651" t="n">
+        <v>0</v>
+      </c>
+      <c r="N651" t="n">
+        <v>0</v>
+      </c>
+      <c r="O651" t="n">
+        <v>0</v>
+      </c>
+      <c r="P651" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q651" t="n">
+        <v>0</v>
+      </c>
+      <c r="R651" t="n">
+        <v>1</v>
+      </c>
+      <c r="S651" t="n">
+        <v>0</v>
+      </c>
+      <c r="T651" t="n">
+        <v>0</v>
+      </c>
+      <c r="U651" t="n">
+        <v>0</v>
+      </c>
+      <c r="V651" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W651" t="n">
+        <v>30</v>
+      </c>
+      <c r="X651" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA vs FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2486524</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>C. DE SOUZA PACHECO | G. JOU COLL | J. CREMO | P. JORGENSEN | S. MICOVIC</t>
+        </is>
+      </c>
+      <c r="D652" t="n">
+        <v>5</v>
+      </c>
+      <c r="E652" t="n">
+        <v>32</v>
+      </c>
+      <c r="F652" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G652" t="n">
+        <v>2</v>
+      </c>
+      <c r="H652" t="n">
+        <v>0</v>
+      </c>
+      <c r="I652" t="n">
+        <v>1</v>
+      </c>
+      <c r="J652" t="n">
+        <v>1</v>
+      </c>
+      <c r="K652" t="n">
+        <v>200</v>
+      </c>
+      <c r="L652" t="n">
+        <v>0</v>
+      </c>
+      <c r="M652" t="n">
+        <v>200</v>
+      </c>
+      <c r="N652" t="n">
+        <v>1</v>
+      </c>
+      <c r="O652" t="n">
+        <v>0</v>
+      </c>
+      <c r="P652" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q652" t="n">
+        <v>0</v>
+      </c>
+      <c r="R652" t="n">
+        <v>1</v>
+      </c>
+      <c r="S652" t="n">
+        <v>0</v>
+      </c>
+      <c r="T652" t="n">
+        <v>0</v>
+      </c>
+      <c r="U652" t="n">
+        <v>0</v>
+      </c>
+      <c r="V652" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W652" t="n">
+        <v>30</v>
+      </c>
+      <c r="X652" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA vs FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2486524</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>C. DE SOUZA PACHECO | I. DIOP GAYE | J. CREMO | P. JORGENSEN | S. MICOVIC</t>
+        </is>
+      </c>
+      <c r="D653" t="n">
+        <v>5</v>
+      </c>
+      <c r="E653" t="n">
+        <v>4</v>
+      </c>
+      <c r="F653" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G653" t="n">
+        <v>0</v>
+      </c>
+      <c r="H653" t="n">
+        <v>0</v>
+      </c>
+      <c r="I653" t="n">
+        <v>0</v>
+      </c>
+      <c r="J653" t="n">
+        <v>1</v>
+      </c>
+      <c r="K653" t="n">
+        <v>0</v>
+      </c>
+      <c r="L653" t="n">
+        <v>0</v>
+      </c>
+      <c r="M653" t="n">
+        <v>0</v>
+      </c>
+      <c r="N653" t="n">
+        <v>0</v>
+      </c>
+      <c r="O653" t="n">
+        <v>0</v>
+      </c>
+      <c r="P653" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q653" t="n">
+        <v>0</v>
+      </c>
+      <c r="R653" t="n">
+        <v>0</v>
+      </c>
+      <c r="S653" t="n">
+        <v>0</v>
+      </c>
+      <c r="T653" t="n">
+        <v>1</v>
+      </c>
+      <c r="U653" t="n">
+        <v>0</v>
+      </c>
+      <c r="V653" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W653" t="n">
+        <v>30</v>
+      </c>
+      <c r="X653" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA vs FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2486524</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>C. DE SOUZA PACHECO | J. CREMO | P. JORGENSEN | S. BARRO | S. MICOVIC</t>
+        </is>
+      </c>
+      <c r="D654" t="n">
+        <v>5</v>
+      </c>
+      <c r="E654" t="n">
+        <v>15</v>
+      </c>
+      <c r="F654" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G654" t="n">
+        <v>0</v>
+      </c>
+      <c r="H654" t="n">
+        <v>3</v>
+      </c>
+      <c r="I654" t="n">
+        <v>0</v>
+      </c>
+      <c r="J654" t="n">
+        <v>1</v>
+      </c>
+      <c r="K654" t="n">
+        <v>0</v>
+      </c>
+      <c r="L654" t="n">
+        <v>300</v>
+      </c>
+      <c r="M654" t="n">
+        <v>0</v>
+      </c>
+      <c r="N654" t="n">
+        <v>0</v>
+      </c>
+      <c r="O654" t="n">
+        <v>0</v>
+      </c>
+      <c r="P654" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q654" t="n">
+        <v>0</v>
+      </c>
+      <c r="R654" t="n">
+        <v>1</v>
+      </c>
+      <c r="S654" t="n">
+        <v>0</v>
+      </c>
+      <c r="T654" t="n">
+        <v>0</v>
+      </c>
+      <c r="U654" t="n">
+        <v>0</v>
+      </c>
+      <c r="V654" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W654" t="n">
+        <v>30</v>
+      </c>
+      <c r="X654" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA vs FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>A. SOLA IDDRISU | E. VICEDO AYALA | E. WEMBI | F. ZURBRIGGEN | S. LITTLESON</t>
+        </is>
+      </c>
+      <c r="D655" t="n">
+        <v>5</v>
+      </c>
+      <c r="E655" t="n">
+        <v>7</v>
+      </c>
+      <c r="F655" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G655" t="n">
+        <v>0</v>
+      </c>
+      <c r="H655" t="n">
+        <v>0</v>
+      </c>
+      <c r="I655" t="n">
+        <v>0</v>
+      </c>
+      <c r="J655" t="n">
+        <v>0</v>
+      </c>
+      <c r="K655" t="n">
+        <v>0</v>
+      </c>
+      <c r="L655" t="n">
+        <v>0</v>
+      </c>
+      <c r="M655" t="n">
+        <v>0</v>
+      </c>
+      <c r="N655" t="n">
+        <v>0</v>
+      </c>
+      <c r="O655" t="n">
+        <v>0</v>
+      </c>
+      <c r="P655" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q655" t="n">
+        <v>0</v>
+      </c>
+      <c r="R655" t="n">
+        <v>0</v>
+      </c>
+      <c r="S655" t="n">
+        <v>0</v>
+      </c>
+      <c r="T655" t="n">
+        <v>0</v>
+      </c>
+      <c r="U655" t="n">
+        <v>0</v>
+      </c>
+      <c r="V655" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W655" t="n">
+        <v>30</v>
+      </c>
+      <c r="X655" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>A. SOLA IDDRISU | E. VICEDO AYALA | F. ZURBRIGGEN | S. LITTLESON | V. ARTEAGA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="D656" t="n">
+        <v>5</v>
+      </c>
+      <c r="E656" t="n">
+        <v>99</v>
+      </c>
+      <c r="F656" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G656" t="n">
+        <v>1</v>
+      </c>
+      <c r="H656" t="n">
+        <v>2</v>
+      </c>
+      <c r="I656" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="J656" t="n">
+        <v>4</v>
+      </c>
+      <c r="K656" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="L656" t="n">
+        <v>50</v>
+      </c>
+      <c r="M656" t="n">
+        <v>-29.51</v>
+      </c>
+      <c r="N656" t="n">
+        <v>3</v>
+      </c>
+      <c r="O656" t="n">
+        <v>2</v>
+      </c>
+      <c r="P656" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q656" t="n">
+        <v>0</v>
+      </c>
+      <c r="R656" t="n">
+        <v>4</v>
+      </c>
+      <c r="S656" t="n">
+        <v>0</v>
+      </c>
+      <c r="T656" t="n">
+        <v>1</v>
+      </c>
+      <c r="U656" t="n">
+        <v>1</v>
+      </c>
+      <c r="V656" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W656" t="n">
+        <v>30</v>
+      </c>
+      <c r="X656" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>A. SOLA IDDRISU | E. VICEDO AYALA | J. CONE | S. LITTLESON | V. ARTEAGA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="D657" t="n">
+        <v>5</v>
+      </c>
+      <c r="E657" t="n">
+        <v>107</v>
+      </c>
+      <c r="F657" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="G657" t="n">
+        <v>4</v>
+      </c>
+      <c r="H657" t="n">
+        <v>5</v>
+      </c>
+      <c r="I657" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J657" t="n">
+        <v>3</v>
+      </c>
+      <c r="K657" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="L657" t="n">
+        <v>166.67</v>
+      </c>
+      <c r="M657" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="N657" t="n">
+        <v>3</v>
+      </c>
+      <c r="O657" t="n">
+        <v>2</v>
+      </c>
+      <c r="P657" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q657" t="n">
+        <v>2</v>
+      </c>
+      <c r="R657" t="n">
+        <v>3</v>
+      </c>
+      <c r="S657" t="n">
+        <v>0</v>
+      </c>
+      <c r="T657" t="n">
+        <v>0</v>
+      </c>
+      <c r="U657" t="n">
+        <v>0</v>
+      </c>
+      <c r="V657" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W657" t="n">
+        <v>30</v>
+      </c>
+      <c r="X657" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>A. SOLA IDDRISU | F. ZURBRIGGEN | N. GALETTE | S. LITTLESON | V. ARTEAGA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>5</v>
+      </c>
+      <c r="E658" t="n">
+        <v>48</v>
+      </c>
+      <c r="F658" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G658" t="n">
+        <v>2</v>
+      </c>
+      <c r="H658" t="n">
+        <v>0</v>
+      </c>
+      <c r="I658" t="n">
+        <v>2</v>
+      </c>
+      <c r="J658" t="n">
+        <v>2</v>
+      </c>
+      <c r="K658" t="n">
+        <v>100</v>
+      </c>
+      <c r="L658" t="n">
+        <v>0</v>
+      </c>
+      <c r="M658" t="n">
+        <v>100</v>
+      </c>
+      <c r="N658" t="n">
+        <v>2</v>
+      </c>
+      <c r="O658" t="n">
+        <v>0</v>
+      </c>
+      <c r="P658" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q658" t="n">
+        <v>0</v>
+      </c>
+      <c r="R658" t="n">
+        <v>2</v>
+      </c>
+      <c r="S658" t="n">
+        <v>0</v>
+      </c>
+      <c r="T658" t="n">
+        <v>0</v>
+      </c>
+      <c r="U658" t="n">
+        <v>0</v>
+      </c>
+      <c r="V658" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W658" t="n">
+        <v>30</v>
+      </c>
+      <c r="X658" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>A. SOLA IDDRISU | J. CONE | N. GALETTE | S. LITTLESON | V. ARTEAGA GONZALEZ</t>
+        </is>
+      </c>
+      <c r="D659" t="n">
+        <v>5</v>
+      </c>
+      <c r="E659" t="n">
+        <v>10</v>
+      </c>
+      <c r="F659" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G659" t="n">
+        <v>0</v>
+      </c>
+      <c r="H659" t="n">
+        <v>0</v>
+      </c>
+      <c r="I659" t="n">
+        <v>0</v>
+      </c>
+      <c r="J659" t="n">
+        <v>0</v>
+      </c>
+      <c r="K659" t="n">
+        <v>0</v>
+      </c>
+      <c r="L659" t="n">
+        <v>0</v>
+      </c>
+      <c r="M659" t="n">
+        <v>0</v>
+      </c>
+      <c r="N659" t="n">
+        <v>0</v>
+      </c>
+      <c r="O659" t="n">
+        <v>0</v>
+      </c>
+      <c r="P659" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q659" t="n">
+        <v>0</v>
+      </c>
+      <c r="R659" t="n">
+        <v>0</v>
+      </c>
+      <c r="S659" t="n">
+        <v>0</v>
+      </c>
+      <c r="T659" t="n">
+        <v>0</v>
+      </c>
+      <c r="U659" t="n">
+        <v>0</v>
+      </c>
+      <c r="V659" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W659" t="n">
+        <v>30</v>
+      </c>
+      <c r="X659" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>E. VICEDO AYALA | E. WEMBI | F. ZURBRIGGEN | J. LOBO MARTORELL | S. LITTLESON</t>
+        </is>
+      </c>
+      <c r="D660" t="n">
+        <v>5</v>
+      </c>
+      <c r="E660" t="n">
+        <v>28</v>
+      </c>
+      <c r="F660" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="G660" t="n">
+        <v>0</v>
+      </c>
+      <c r="H660" t="n">
+        <v>1</v>
+      </c>
+      <c r="I660" t="n">
+        <v>1</v>
+      </c>
+      <c r="J660" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="K660" t="n">
+        <v>0</v>
+      </c>
+      <c r="L660" t="n">
+        <v>53.19</v>
+      </c>
+      <c r="M660" t="n">
+        <v>-53.19</v>
+      </c>
+      <c r="N660" t="n">
+        <v>2</v>
+      </c>
+      <c r="O660" t="n">
+        <v>0</v>
+      </c>
+      <c r="P660" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q660" t="n">
+        <v>1</v>
+      </c>
+      <c r="R660" t="n">
+        <v>0</v>
+      </c>
+      <c r="S660" t="n">
+        <v>2</v>
+      </c>
+      <c r="T660" t="n">
+        <v>1</v>
+      </c>
+      <c r="U660" t="n">
+        <v>0</v>
+      </c>
+      <c r="V660" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W660" t="n">
+        <v>30</v>
+      </c>
+      <c r="X660" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>A. WINTERING | J. VRANKIC | M. ARMUS | M. KAMBA | T. BORG</t>
+        </is>
+      </c>
+      <c r="D661" t="n">
+        <v>5</v>
+      </c>
+      <c r="E661" t="n">
+        <v>10</v>
+      </c>
+      <c r="F661" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G661" t="n">
+        <v>0</v>
+      </c>
+      <c r="H661" t="n">
+        <v>0</v>
+      </c>
+      <c r="I661" t="n">
+        <v>0</v>
+      </c>
+      <c r="J661" t="n">
+        <v>0</v>
+      </c>
+      <c r="K661" t="n">
+        <v>0</v>
+      </c>
+      <c r="L661" t="n">
+        <v>0</v>
+      </c>
+      <c r="M661" t="n">
+        <v>0</v>
+      </c>
+      <c r="N661" t="n">
+        <v>0</v>
+      </c>
+      <c r="O661" t="n">
+        <v>0</v>
+      </c>
+      <c r="P661" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q661" t="n">
+        <v>0</v>
+      </c>
+      <c r="R661" t="n">
+        <v>0</v>
+      </c>
+      <c r="S661" t="n">
+        <v>0</v>
+      </c>
+      <c r="T661" t="n">
+        <v>0</v>
+      </c>
+      <c r="U661" t="n">
+        <v>0</v>
+      </c>
+      <c r="V661" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W661" t="n">
+        <v>30</v>
+      </c>
+      <c r="X661" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>A. WINTERING | J. VRANKIC | M. ARMUS | T. BORG | X. OROZ URIA</t>
+        </is>
+      </c>
+      <c r="D662" t="n">
+        <v>5</v>
+      </c>
+      <c r="E662" t="n">
+        <v>48</v>
+      </c>
+      <c r="F662" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G662" t="n">
+        <v>0</v>
+      </c>
+      <c r="H662" t="n">
+        <v>2</v>
+      </c>
+      <c r="I662" t="n">
+        <v>2</v>
+      </c>
+      <c r="J662" t="n">
+        <v>2</v>
+      </c>
+      <c r="K662" t="n">
+        <v>0</v>
+      </c>
+      <c r="L662" t="n">
+        <v>100</v>
+      </c>
+      <c r="M662" t="n">
+        <v>-100</v>
+      </c>
+      <c r="N662" t="n">
+        <v>2</v>
+      </c>
+      <c r="O662" t="n">
+        <v>0</v>
+      </c>
+      <c r="P662" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q662" t="n">
+        <v>0</v>
+      </c>
+      <c r="R662" t="n">
+        <v>2</v>
+      </c>
+      <c r="S662" t="n">
+        <v>0</v>
+      </c>
+      <c r="T662" t="n">
+        <v>0</v>
+      </c>
+      <c r="U662" t="n">
+        <v>0</v>
+      </c>
+      <c r="V662" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W662" t="n">
+        <v>30</v>
+      </c>
+      <c r="X662" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2486520</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>A. WINTERING | J. VRANKIC | M. KAMBA | T. BORG | V. VUCETIC</t>
+        </is>
+      </c>
+      <c r="D663" t="n">
+        <v>5</v>
+      </c>
+      <c r="E663" t="n">
+        <v>241</v>
+      </c>
+      <c r="F663" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G663" t="n">
+        <v>8</v>
+      </c>
+      <c r="H663" t="n">
+        <v>5</v>
+      </c>
+      <c r="I663" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="J663" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="K663" t="n">
+        <v>90.09</v>
+      </c>
+      <c r="L663" t="n">
+        <v>64.43000000000001</v>
+      </c>
+      <c r="M663" t="n">
+        <v>25.66</v>
+      </c>
+      <c r="N663" t="n">
+        <v>7</v>
+      </c>
+      <c r="O663" t="n">
+        <v>2</v>
+      </c>
+      <c r="P663" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q663" t="n">
+        <v>1</v>
+      </c>
+      <c r="R663" t="n">
+        <v>8</v>
+      </c>
+      <c r="S663" t="n">
+        <v>4</v>
+      </c>
+      <c r="T663" t="n">
+        <v>1</v>
+      </c>
+      <c r="U663" t="n">
+        <v>3</v>
+      </c>
+      <c r="V663" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W663" t="n">
+        <v>30</v>
+      </c>
+      <c r="X663" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA vs HESTIA MENORCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2486523</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>A. FAURE RIBES | D. DUSCAK | G. PARHAM II | M. TOWNES VILLAR | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D664" t="n">
+        <v>5</v>
+      </c>
+      <c r="E664" t="n">
+        <v>70</v>
+      </c>
+      <c r="F664" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="G664" t="n">
+        <v>2</v>
+      </c>
+      <c r="H664" t="n">
+        <v>4</v>
+      </c>
+      <c r="I664" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="J664" t="n">
+        <v>2</v>
+      </c>
+      <c r="K664" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="L664" t="n">
+        <v>200</v>
+      </c>
+      <c r="M664" t="n">
+        <v>-130.56</v>
+      </c>
+      <c r="N664" t="n">
+        <v>1</v>
+      </c>
+      <c r="O664" t="n">
+        <v>2</v>
+      </c>
+      <c r="P664" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q664" t="n">
+        <v>0</v>
+      </c>
+      <c r="R664" t="n">
+        <v>2</v>
+      </c>
+      <c r="S664" t="n">
+        <v>0</v>
+      </c>
+      <c r="T664" t="n">
+        <v>1</v>
+      </c>
+      <c r="U664" t="n">
+        <v>1</v>
+      </c>
+      <c r="V664" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W664" t="n">
+        <v>30</v>
+      </c>
+      <c r="X664" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2486523</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>D. DUSCAK | D. SHELIST | F. NWAOKORIE | G. PARHAM II | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D665" t="n">
+        <v>5</v>
+      </c>
+      <c r="E665" t="n">
+        <v>111</v>
+      </c>
+      <c r="F665" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G665" t="n">
+        <v>1</v>
+      </c>
+      <c r="H665" t="n">
+        <v>0</v>
+      </c>
+      <c r="I665" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="J665" t="n">
+        <v>3</v>
+      </c>
+      <c r="K665" t="n">
+        <v>40.98</v>
+      </c>
+      <c r="L665" t="n">
+        <v>0</v>
+      </c>
+      <c r="M665" t="n">
+        <v>40.98</v>
+      </c>
+      <c r="N665" t="n">
+        <v>2</v>
+      </c>
+      <c r="O665" t="n">
+        <v>1</v>
+      </c>
+      <c r="P665" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q665" t="n">
+        <v>1</v>
+      </c>
+      <c r="R665" t="n">
+        <v>2</v>
+      </c>
+      <c r="S665" t="n">
+        <v>0</v>
+      </c>
+      <c r="T665" t="n">
+        <v>2</v>
+      </c>
+      <c r="U665" t="n">
+        <v>1</v>
+      </c>
+      <c r="V665" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W665" t="n">
+        <v>30</v>
+      </c>
+      <c r="X665" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2486523</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>D. DUSCAK | D. SHELIST | G. PARHAM II | M. TOWNES VILLAR | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D666" t="n">
+        <v>5</v>
+      </c>
+      <c r="E666" t="n">
+        <v>51</v>
+      </c>
+      <c r="F666" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G666" t="n">
+        <v>0</v>
+      </c>
+      <c r="H666" t="n">
+        <v>0</v>
+      </c>
+      <c r="I666" t="n">
+        <v>2</v>
+      </c>
+      <c r="J666" t="n">
+        <v>1</v>
+      </c>
+      <c r="K666" t="n">
+        <v>0</v>
+      </c>
+      <c r="L666" t="n">
+        <v>0</v>
+      </c>
+      <c r="M666" t="n">
+        <v>0</v>
+      </c>
+      <c r="N666" t="n">
+        <v>2</v>
+      </c>
+      <c r="O666" t="n">
+        <v>0</v>
+      </c>
+      <c r="P666" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q666" t="n">
+        <v>0</v>
+      </c>
+      <c r="R666" t="n">
+        <v>1</v>
+      </c>
+      <c r="S666" t="n">
+        <v>0</v>
+      </c>
+      <c r="T666" t="n">
+        <v>0</v>
+      </c>
+      <c r="U666" t="n">
+        <v>0</v>
+      </c>
+      <c r="V666" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W666" t="n">
+        <v>30</v>
+      </c>
+      <c r="X666" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2486523</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>D. SHELIST | F. NWAOKORIE | G. PARHAM II | M. TOWNES VILLAR | R. LOBACO MUÑOZ</t>
+        </is>
+      </c>
+      <c r="D667" t="n">
+        <v>5</v>
+      </c>
+      <c r="E667" t="n">
+        <v>31</v>
+      </c>
+      <c r="F667" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G667" t="n">
+        <v>0</v>
+      </c>
+      <c r="H667" t="n">
+        <v>2</v>
+      </c>
+      <c r="I667" t="n">
+        <v>1</v>
+      </c>
+      <c r="J667" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="K667" t="n">
+        <v>0</v>
+      </c>
+      <c r="L667" t="n">
+        <v>106.38</v>
+      </c>
+      <c r="M667" t="n">
+        <v>-106.38</v>
+      </c>
+      <c r="N667" t="n">
+        <v>0</v>
+      </c>
+      <c r="O667" t="n">
+        <v>0</v>
+      </c>
+      <c r="P667" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q667" t="n">
+        <v>0</v>
+      </c>
+      <c r="R667" t="n">
+        <v>1</v>
+      </c>
+      <c r="S667" t="n">
+        <v>2</v>
+      </c>
+      <c r="T667" t="n">
+        <v>0</v>
+      </c>
+      <c r="U667" t="n">
+        <v>0</v>
+      </c>
+      <c r="V667" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W667" t="n">
+        <v>30</v>
+      </c>
+      <c r="X667" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2486523</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>H. LOPEZ BARRANTES | J. GRANGER | L. GIOVANNETTI | P. GARINO GULLOTTA | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D668" t="n">
+        <v>5</v>
+      </c>
+      <c r="E668" t="n">
+        <v>111</v>
+      </c>
+      <c r="F668" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G668" t="n">
+        <v>0</v>
+      </c>
+      <c r="H668" t="n">
+        <v>1</v>
+      </c>
+      <c r="I668" t="n">
+        <v>3</v>
+      </c>
+      <c r="J668" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="K668" t="n">
+        <v>0</v>
+      </c>
+      <c r="L668" t="n">
+        <v>40.98</v>
+      </c>
+      <c r="M668" t="n">
+        <v>-40.98</v>
+      </c>
+      <c r="N668" t="n">
+        <v>2</v>
+      </c>
+      <c r="O668" t="n">
+        <v>0</v>
+      </c>
+      <c r="P668" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q668" t="n">
+        <v>1</v>
+      </c>
+      <c r="R668" t="n">
+        <v>2</v>
+      </c>
+      <c r="S668" t="n">
+        <v>1</v>
+      </c>
+      <c r="T668" t="n">
+        <v>1</v>
+      </c>
+      <c r="U668" t="n">
+        <v>1</v>
+      </c>
+      <c r="V668" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W668" t="n">
+        <v>30</v>
+      </c>
+      <c r="X668" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2486523</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>H. LOPEZ BARRANTES | J. GRANGER | P. GARINO GULLOTTA | S. SALIN | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D669" t="n">
+        <v>5</v>
+      </c>
+      <c r="E669" t="n">
+        <v>8</v>
+      </c>
+      <c r="F669" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G669" t="n">
+        <v>0</v>
+      </c>
+      <c r="H669" t="n">
+        <v>0</v>
+      </c>
+      <c r="I669" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J669" t="n">
+        <v>0</v>
+      </c>
+      <c r="K669" t="n">
+        <v>0</v>
+      </c>
+      <c r="L669" t="n">
+        <v>0</v>
+      </c>
+      <c r="M669" t="n">
+        <v>0</v>
+      </c>
+      <c r="N669" t="n">
+        <v>0</v>
+      </c>
+      <c r="O669" t="n">
+        <v>2</v>
+      </c>
+      <c r="P669" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q669" t="n">
+        <v>0</v>
+      </c>
+      <c r="R669" t="n">
+        <v>0</v>
+      </c>
+      <c r="S669" t="n">
+        <v>0</v>
+      </c>
+      <c r="T669" t="n">
+        <v>0</v>
+      </c>
+      <c r="U669" t="n">
+        <v>0</v>
+      </c>
+      <c r="V669" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W669" t="n">
+        <v>30</v>
+      </c>
+      <c r="X669" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2486523</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>J. GRANGER | L. GIOVANNETTI | L. NWOGBO | P. GARINO GULLOTTA | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D670" t="n">
+        <v>5</v>
+      </c>
+      <c r="E670" t="n">
+        <v>8</v>
+      </c>
+      <c r="F670" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G670" t="n">
+        <v>0</v>
+      </c>
+      <c r="H670" t="n">
+        <v>0</v>
+      </c>
+      <c r="I670" t="n">
+        <v>1</v>
+      </c>
+      <c r="J670" t="n">
+        <v>0</v>
+      </c>
+      <c r="K670" t="n">
+        <v>0</v>
+      </c>
+      <c r="L670" t="n">
+        <v>0</v>
+      </c>
+      <c r="M670" t="n">
+        <v>0</v>
+      </c>
+      <c r="N670" t="n">
+        <v>0</v>
+      </c>
+      <c r="O670" t="n">
+        <v>0</v>
+      </c>
+      <c r="P670" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q670" t="n">
+        <v>0</v>
+      </c>
+      <c r="R670" t="n">
+        <v>0</v>
+      </c>
+      <c r="S670" t="n">
+        <v>0</v>
+      </c>
+      <c r="T670" t="n">
+        <v>0</v>
+      </c>
+      <c r="U670" t="n">
+        <v>0</v>
+      </c>
+      <c r="V670" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W670" t="n">
+        <v>30</v>
+      </c>
+      <c r="X670" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2486523</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>J. GRANGER | L. NWOGBO | P. GARINO GULLOTTA | S. SALIN | T. MC GREW</t>
+        </is>
+      </c>
+      <c r="D671" t="n">
+        <v>5</v>
+      </c>
+      <c r="E671" t="n">
+        <v>136</v>
+      </c>
+      <c r="F671" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="G671" t="n">
+        <v>6</v>
+      </c>
+      <c r="H671" t="n">
+        <v>2</v>
+      </c>
+      <c r="I671" t="n">
+        <v>3</v>
+      </c>
+      <c r="J671" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="K671" t="n">
+        <v>200</v>
+      </c>
+      <c r="L671" t="n">
+        <v>34.01</v>
+      </c>
+      <c r="M671" t="n">
+        <v>165.99</v>
+      </c>
+      <c r="N671" t="n">
+        <v>4</v>
+      </c>
+      <c r="O671" t="n">
+        <v>0</v>
+      </c>
+      <c r="P671" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q671" t="n">
+        <v>1</v>
+      </c>
+      <c r="R671" t="n">
+        <v>3</v>
+      </c>
+      <c r="S671" t="n">
+        <v>2</v>
+      </c>
+      <c r="T671" t="n">
+        <v>2</v>
+      </c>
+      <c r="U671" t="n">
+        <v>0</v>
+      </c>
+      <c r="V671" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W671" t="n">
+        <v>30</v>
+      </c>
+      <c r="X671" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO vs MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2486519</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>A. SCARIOLO ARES | J. BOCCA | L. BRACEY | O. MATULIONIS | S. NIANG BEYE</t>
+        </is>
+      </c>
+      <c r="D672" t="n">
+        <v>5</v>
+      </c>
+      <c r="E672" t="n">
+        <v>46</v>
+      </c>
+      <c r="F672" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G672" t="n">
+        <v>0</v>
+      </c>
+      <c r="H672" t="n">
+        <v>0</v>
+      </c>
+      <c r="I672" t="n">
+        <v>0</v>
+      </c>
+      <c r="J672" t="n">
+        <v>1</v>
+      </c>
+      <c r="K672" t="n">
+        <v>0</v>
+      </c>
+      <c r="L672" t="n">
+        <v>0</v>
+      </c>
+      <c r="M672" t="n">
+        <v>0</v>
+      </c>
+      <c r="N672" t="n">
+        <v>1</v>
+      </c>
+      <c r="O672" t="n">
+        <v>0</v>
+      </c>
+      <c r="P672" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q672" t="n">
+        <v>1</v>
+      </c>
+      <c r="R672" t="n">
+        <v>1</v>
+      </c>
+      <c r="S672" t="n">
+        <v>0</v>
+      </c>
+      <c r="T672" t="n">
+        <v>0</v>
+      </c>
+      <c r="U672" t="n">
+        <v>0</v>
+      </c>
+      <c r="V672" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W672" t="n">
+        <v>30</v>
+      </c>
+      <c r="X672" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2486519</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>A. SCARIOLO ARES | J. BOCCA | L. CAPALBO | O. MATULIONIS | S. NIANG BEYE</t>
+        </is>
+      </c>
+      <c r="D673" t="n">
+        <v>5</v>
+      </c>
+      <c r="E673" t="n">
+        <v>6</v>
+      </c>
+      <c r="F673" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G673" t="n">
+        <v>0</v>
+      </c>
+      <c r="H673" t="n">
+        <v>2</v>
+      </c>
+      <c r="I673" t="n">
+        <v>1</v>
+      </c>
+      <c r="J673" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K673" t="n">
+        <v>0</v>
+      </c>
+      <c r="L673" t="n">
+        <v>227.27</v>
+      </c>
+      <c r="M673" t="n">
+        <v>-227.27</v>
+      </c>
+      <c r="N673" t="n">
+        <v>0</v>
+      </c>
+      <c r="O673" t="n">
+        <v>0</v>
+      </c>
+      <c r="P673" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q673" t="n">
+        <v>0</v>
+      </c>
+      <c r="R673" t="n">
+        <v>0</v>
+      </c>
+      <c r="S673" t="n">
+        <v>2</v>
+      </c>
+      <c r="T673" t="n">
+        <v>0</v>
+      </c>
+      <c r="U673" t="n">
+        <v>0</v>
+      </c>
+      <c r="V673" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W673" t="n">
+        <v>30</v>
+      </c>
+      <c r="X673" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2486519</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>J. BOCCA | L. BRACEY | L. CAPALBO | L. SMITH | O. MATULIONIS</t>
+        </is>
+      </c>
+      <c r="D674" t="n">
+        <v>5</v>
+      </c>
+      <c r="E674" t="n">
+        <v>66</v>
+      </c>
+      <c r="F674" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G674" t="n">
+        <v>0</v>
+      </c>
+      <c r="H674" t="n">
+        <v>3</v>
+      </c>
+      <c r="I674" t="n">
+        <v>1</v>
+      </c>
+      <c r="J674" t="n">
+        <v>0</v>
+      </c>
+      <c r="K674" t="n">
+        <v>0</v>
+      </c>
+      <c r="L674" t="n">
+        <v>0</v>
+      </c>
+      <c r="M674" t="n">
+        <v>0</v>
+      </c>
+      <c r="N674" t="n">
+        <v>2</v>
+      </c>
+      <c r="O674" t="n">
+        <v>0</v>
+      </c>
+      <c r="P674" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q674" t="n">
+        <v>1</v>
+      </c>
+      <c r="R674" t="n">
+        <v>2</v>
+      </c>
+      <c r="S674" t="n">
+        <v>0</v>
+      </c>
+      <c r="T674" t="n">
+        <v>0</v>
+      </c>
+      <c r="U674" t="n">
+        <v>2</v>
+      </c>
+      <c r="V674" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W674" t="n">
+        <v>30</v>
+      </c>
+      <c r="X674" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2486519</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>L. BRACEY | L. CAPALBO | L. SMITH | O. MATULIONIS | S. NIANG BEYE</t>
+        </is>
+      </c>
+      <c r="D675" t="n">
+        <v>5</v>
+      </c>
+      <c r="E675" t="n">
+        <v>161</v>
+      </c>
+      <c r="F675" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="G675" t="n">
+        <v>4</v>
+      </c>
+      <c r="H675" t="n">
+        <v>5</v>
+      </c>
+      <c r="I675" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="J675" t="n">
+        <v>5</v>
+      </c>
+      <c r="K675" t="n">
+        <v>103.09</v>
+      </c>
+      <c r="L675" t="n">
+        <v>100</v>
+      </c>
+      <c r="M675" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="N675" t="n">
+        <v>1</v>
+      </c>
+      <c r="O675" t="n">
+        <v>2</v>
+      </c>
+      <c r="P675" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q675" t="n">
+        <v>1</v>
+      </c>
+      <c r="R675" t="n">
+        <v>4</v>
+      </c>
+      <c r="S675" t="n">
+        <v>0</v>
+      </c>
+      <c r="T675" t="n">
+        <v>1</v>
+      </c>
+      <c r="U675" t="n">
+        <v>0</v>
+      </c>
+      <c r="V675" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W675" t="n">
+        <v>30</v>
+      </c>
+      <c r="X675" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2486519</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | A. MARTIN MARIN | C. POLYNICE | I. RIVERA CARROLL | J. LOPEZ SANTANA</t>
+        </is>
+      </c>
+      <c r="D676" t="n">
+        <v>5</v>
+      </c>
+      <c r="E676" t="n">
+        <v>34</v>
+      </c>
+      <c r="F676" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G676" t="n">
+        <v>0</v>
+      </c>
+      <c r="H676" t="n">
+        <v>0</v>
+      </c>
+      <c r="I676" t="n">
+        <v>1</v>
+      </c>
+      <c r="J676" t="n">
+        <v>0</v>
+      </c>
+      <c r="K676" t="n">
+        <v>0</v>
+      </c>
+      <c r="L676" t="n">
+        <v>0</v>
+      </c>
+      <c r="M676" t="n">
+        <v>0</v>
+      </c>
+      <c r="N676" t="n">
+        <v>1</v>
+      </c>
+      <c r="O676" t="n">
+        <v>0</v>
+      </c>
+      <c r="P676" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q676" t="n">
+        <v>0</v>
+      </c>
+      <c r="R676" t="n">
+        <v>1</v>
+      </c>
+      <c r="S676" t="n">
+        <v>0</v>
+      </c>
+      <c r="T676" t="n">
+        <v>0</v>
+      </c>
+      <c r="U676" t="n">
+        <v>1</v>
+      </c>
+      <c r="V676" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W676" t="n">
+        <v>30</v>
+      </c>
+      <c r="X676" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2486519</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | A. MARTIN MARIN | I. RIVERA CARROLL | K. WEBSTER | S. SVEJCAR</t>
+        </is>
+      </c>
+      <c r="D677" t="n">
+        <v>5</v>
+      </c>
+      <c r="E677" t="n">
+        <v>6</v>
+      </c>
+      <c r="F677" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G677" t="n">
+        <v>0</v>
+      </c>
+      <c r="H677" t="n">
+        <v>0</v>
+      </c>
+      <c r="I677" t="n">
+        <v>1</v>
+      </c>
+      <c r="J677" t="n">
+        <v>1</v>
+      </c>
+      <c r="K677" t="n">
+        <v>0</v>
+      </c>
+      <c r="L677" t="n">
+        <v>0</v>
+      </c>
+      <c r="M677" t="n">
+        <v>0</v>
+      </c>
+      <c r="N677" t="n">
+        <v>0</v>
+      </c>
+      <c r="O677" t="n">
+        <v>0</v>
+      </c>
+      <c r="P677" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q677" t="n">
+        <v>0</v>
+      </c>
+      <c r="R677" t="n">
+        <v>0</v>
+      </c>
+      <c r="S677" t="n">
+        <v>0</v>
+      </c>
+      <c r="T677" t="n">
+        <v>1</v>
+      </c>
+      <c r="U677" t="n">
+        <v>0</v>
+      </c>
+      <c r="V677" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W677" t="n">
+        <v>30</v>
+      </c>
+      <c r="X677" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2486519</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>A. GARUBA ALARI | A. MARTIN MARIN | K. WEBSTER | S. SVEJCAR | V. FAVERANI TATSCH</t>
+        </is>
+      </c>
+      <c r="D678" t="n">
+        <v>5</v>
+      </c>
+      <c r="E678" t="n">
+        <v>239</v>
+      </c>
+      <c r="F678" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="G678" t="n">
+        <v>10</v>
+      </c>
+      <c r="H678" t="n">
+        <v>4</v>
+      </c>
+      <c r="I678" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="J678" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="K678" t="n">
+        <v>204.92</v>
+      </c>
+      <c r="L678" t="n">
+        <v>81.97</v>
+      </c>
+      <c r="M678" t="n">
+        <v>122.95</v>
+      </c>
+      <c r="N678" t="n">
+        <v>6</v>
+      </c>
+      <c r="O678" t="n">
+        <v>2</v>
+      </c>
+      <c r="P678" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q678" t="n">
+        <v>2</v>
+      </c>
+      <c r="R678" t="n">
+        <v>3</v>
+      </c>
+      <c r="S678" t="n">
+        <v>2</v>
+      </c>
+      <c r="T678" t="n">
+        <v>3</v>
+      </c>
+      <c r="U678" t="n">
+        <v>2</v>
+      </c>
+      <c r="V678" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W678" t="n">
+        <v>30</v>
+      </c>
+      <c r="X678" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB vs FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>A. MARTINEZ CLARIANA | B. PREPELIC | J. PERIS CRESPO | J. VAN ZEGEREN | T. NASPLER PERAIRE</t>
+        </is>
+      </c>
+      <c r="D679" t="n">
+        <v>5</v>
+      </c>
+      <c r="E679" t="n">
+        <v>11</v>
+      </c>
+      <c r="F679" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G679" t="n">
+        <v>0</v>
+      </c>
+      <c r="H679" t="n">
+        <v>2</v>
+      </c>
+      <c r="I679" t="n">
+        <v>0</v>
+      </c>
+      <c r="J679" t="n">
+        <v>1</v>
+      </c>
+      <c r="K679" t="n">
+        <v>0</v>
+      </c>
+      <c r="L679" t="n">
+        <v>200</v>
+      </c>
+      <c r="M679" t="n">
+        <v>0</v>
+      </c>
+      <c r="N679" t="n">
+        <v>0</v>
+      </c>
+      <c r="O679" t="n">
+        <v>0</v>
+      </c>
+      <c r="P679" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q679" t="n">
+        <v>0</v>
+      </c>
+      <c r="R679" t="n">
+        <v>1</v>
+      </c>
+      <c r="S679" t="n">
+        <v>0</v>
+      </c>
+      <c r="T679" t="n">
+        <v>0</v>
+      </c>
+      <c r="U679" t="n">
+        <v>0</v>
+      </c>
+      <c r="V679" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W679" t="n">
+        <v>30</v>
+      </c>
+      <c r="X679" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>B. PREPELIC | J. ROUND | O. LO | T. NASPLER PERAIRE | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D680" t="n">
+        <v>5</v>
+      </c>
+      <c r="E680" t="n">
+        <v>91</v>
+      </c>
+      <c r="F680" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="G680" t="n">
+        <v>4</v>
+      </c>
+      <c r="H680" t="n">
+        <v>0</v>
+      </c>
+      <c r="I680" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J680" t="n">
+        <v>2</v>
+      </c>
+      <c r="K680" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="L680" t="n">
+        <v>0</v>
+      </c>
+      <c r="M680" t="n">
+        <v>212.77</v>
+      </c>
+      <c r="N680" t="n">
+        <v>2</v>
+      </c>
+      <c r="O680" t="n">
+        <v>2</v>
+      </c>
+      <c r="P680" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q680" t="n">
+        <v>2</v>
+      </c>
+      <c r="R680" t="n">
+        <v>2</v>
+      </c>
+      <c r="S680" t="n">
+        <v>0</v>
+      </c>
+      <c r="T680" t="n">
+        <v>0</v>
+      </c>
+      <c r="U680" t="n">
+        <v>0</v>
+      </c>
+      <c r="V680" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W680" t="n">
+        <v>30</v>
+      </c>
+      <c r="X680" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>C. ROGERS | J. PERIS CRESPO | J. ROUND | O. LO | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D681" t="n">
+        <v>5</v>
+      </c>
+      <c r="E681" t="n">
+        <v>17</v>
+      </c>
+      <c r="F681" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G681" t="n">
+        <v>0</v>
+      </c>
+      <c r="H681" t="n">
+        <v>3</v>
+      </c>
+      <c r="I681" t="n">
+        <v>2</v>
+      </c>
+      <c r="J681" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="K681" t="n">
+        <v>0</v>
+      </c>
+      <c r="L681" t="n">
+        <v>394.74</v>
+      </c>
+      <c r="M681" t="n">
+        <v>-394.74</v>
+      </c>
+      <c r="N681" t="n">
+        <v>1</v>
+      </c>
+      <c r="O681" t="n">
+        <v>0</v>
+      </c>
+      <c r="P681" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q681" t="n">
+        <v>0</v>
+      </c>
+      <c r="R681" t="n">
+        <v>0</v>
+      </c>
+      <c r="S681" t="n">
+        <v>4</v>
+      </c>
+      <c r="T681" t="n">
+        <v>0</v>
+      </c>
+      <c r="U681" t="n">
+        <v>1</v>
+      </c>
+      <c r="V681" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W681" t="n">
+        <v>30</v>
+      </c>
+      <c r="X681" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>C. ROGERS | J. PERIS CRESPO | J. VAN ZEGEREN | S. THRASTARSON | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D682" t="n">
+        <v>5</v>
+      </c>
+      <c r="E682" t="n">
+        <v>17</v>
+      </c>
+      <c r="F682" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G682" t="n">
+        <v>3</v>
+      </c>
+      <c r="H682" t="n">
+        <v>1</v>
+      </c>
+      <c r="I682" t="n">
+        <v>1</v>
+      </c>
+      <c r="J682" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K682" t="n">
+        <v>300</v>
+      </c>
+      <c r="L682" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="M682" t="n">
+        <v>186.36</v>
+      </c>
+      <c r="N682" t="n">
+        <v>2</v>
+      </c>
+      <c r="O682" t="n">
+        <v>0</v>
+      </c>
+      <c r="P682" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q682" t="n">
+        <v>1</v>
+      </c>
+      <c r="R682" t="n">
+        <v>0</v>
+      </c>
+      <c r="S682" t="n">
+        <v>2</v>
+      </c>
+      <c r="T682" t="n">
+        <v>0</v>
+      </c>
+      <c r="U682" t="n">
+        <v>0</v>
+      </c>
+      <c r="V682" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W682" t="n">
+        <v>30</v>
+      </c>
+      <c r="X682" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>C. ROGERS | J. PERIS CRESPO | O. LO | S. THRASTARSON | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D683" t="n">
+        <v>5</v>
+      </c>
+      <c r="E683" t="n">
+        <v>53</v>
+      </c>
+      <c r="F683" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G683" t="n">
+        <v>2</v>
+      </c>
+      <c r="H683" t="n">
+        <v>1</v>
+      </c>
+      <c r="I683" t="n">
+        <v>2</v>
+      </c>
+      <c r="J683" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K683" t="n">
+        <v>100</v>
+      </c>
+      <c r="L683" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="M683" t="n">
+        <v>-13.64</v>
+      </c>
+      <c r="N683" t="n">
+        <v>3</v>
+      </c>
+      <c r="O683" t="n">
+        <v>0</v>
+      </c>
+      <c r="P683" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q683" t="n">
+        <v>1</v>
+      </c>
+      <c r="R683" t="n">
+        <v>1</v>
+      </c>
+      <c r="S683" t="n">
+        <v>2</v>
+      </c>
+      <c r="T683" t="n">
+        <v>0</v>
+      </c>
+      <c r="U683" t="n">
+        <v>1</v>
+      </c>
+      <c r="V683" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W683" t="n">
+        <v>30</v>
+      </c>
+      <c r="X683" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>C. ROGERS | J. VAN ZEGEREN | S. THRASTARSON | T. NASPLER PERAIRE | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D684" t="n">
+        <v>5</v>
+      </c>
+      <c r="E684" t="n">
+        <v>58</v>
+      </c>
+      <c r="F684" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G684" t="n">
+        <v>0</v>
+      </c>
+      <c r="H684" t="n">
+        <v>6</v>
+      </c>
+      <c r="I684" t="n">
+        <v>1</v>
+      </c>
+      <c r="J684" t="n">
+        <v>2</v>
+      </c>
+      <c r="K684" t="n">
+        <v>0</v>
+      </c>
+      <c r="L684" t="n">
+        <v>300</v>
+      </c>
+      <c r="M684" t="n">
+        <v>-300</v>
+      </c>
+      <c r="N684" t="n">
+        <v>1</v>
+      </c>
+      <c r="O684" t="n">
+        <v>0</v>
+      </c>
+      <c r="P684" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q684" t="n">
+        <v>0</v>
+      </c>
+      <c r="R684" t="n">
+        <v>2</v>
+      </c>
+      <c r="S684" t="n">
+        <v>0</v>
+      </c>
+      <c r="T684" t="n">
+        <v>0</v>
+      </c>
+      <c r="U684" t="n">
+        <v>0</v>
+      </c>
+      <c r="V684" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W684" t="n">
+        <v>30</v>
+      </c>
+      <c r="X684" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>C. ROGERS | O. LO | S. THRASTARSON | T. NASPLER PERAIRE | T. ROBERTS</t>
+        </is>
+      </c>
+      <c r="D685" t="n">
+        <v>5</v>
+      </c>
+      <c r="E685" t="n">
+        <v>34</v>
+      </c>
+      <c r="F685" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G685" t="n">
+        <v>0</v>
+      </c>
+      <c r="H685" t="n">
+        <v>2</v>
+      </c>
+      <c r="I685" t="n">
+        <v>0</v>
+      </c>
+      <c r="J685" t="n">
+        <v>1</v>
+      </c>
+      <c r="K685" t="n">
+        <v>0</v>
+      </c>
+      <c r="L685" t="n">
+        <v>200</v>
+      </c>
+      <c r="M685" t="n">
+        <v>0</v>
+      </c>
+      <c r="N685" t="n">
+        <v>0</v>
+      </c>
+      <c r="O685" t="n">
+        <v>0</v>
+      </c>
+      <c r="P685" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q685" t="n">
+        <v>0</v>
+      </c>
+      <c r="R685" t="n">
+        <v>1</v>
+      </c>
+      <c r="S685" t="n">
+        <v>0</v>
+      </c>
+      <c r="T685" t="n">
+        <v>0</v>
+      </c>
+      <c r="U685" t="n">
+        <v>0</v>
+      </c>
+      <c r="V685" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W685" t="n">
+        <v>30</v>
+      </c>
+      <c r="X685" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | I. CRUZ UCEDA | J. GARCIA SANCHEZ | M. CAICEDO SANCHEZ | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D686" t="n">
+        <v>5</v>
+      </c>
+      <c r="E686" t="n">
+        <v>34</v>
+      </c>
+      <c r="F686" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G686" t="n">
+        <v>2</v>
+      </c>
+      <c r="H686" t="n">
+        <v>0</v>
+      </c>
+      <c r="I686" t="n">
+        <v>1</v>
+      </c>
+      <c r="J686" t="n">
+        <v>0</v>
+      </c>
+      <c r="K686" t="n">
+        <v>200</v>
+      </c>
+      <c r="L686" t="n">
+        <v>0</v>
+      </c>
+      <c r="M686" t="n">
+        <v>0</v>
+      </c>
+      <c r="N686" t="n">
+        <v>1</v>
+      </c>
+      <c r="O686" t="n">
+        <v>0</v>
+      </c>
+      <c r="P686" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q686" t="n">
+        <v>0</v>
+      </c>
+      <c r="R686" t="n">
+        <v>0</v>
+      </c>
+      <c r="S686" t="n">
+        <v>0</v>
+      </c>
+      <c r="T686" t="n">
+        <v>0</v>
+      </c>
+      <c r="U686" t="n">
+        <v>0</v>
+      </c>
+      <c r="V686" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W686" t="n">
+        <v>30</v>
+      </c>
+      <c r="X686" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | I. CRUZ UCEDA | M. CAICEDO SANCHEZ | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D687" t="n">
+        <v>5</v>
+      </c>
+      <c r="E687" t="n">
+        <v>33</v>
+      </c>
+      <c r="F687" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G687" t="n">
+        <v>0</v>
+      </c>
+      <c r="H687" t="n">
+        <v>2</v>
+      </c>
+      <c r="I687" t="n">
+        <v>0</v>
+      </c>
+      <c r="J687" t="n">
+        <v>1</v>
+      </c>
+      <c r="K687" t="n">
+        <v>0</v>
+      </c>
+      <c r="L687" t="n">
+        <v>200</v>
+      </c>
+      <c r="M687" t="n">
+        <v>0</v>
+      </c>
+      <c r="N687" t="n">
+        <v>1</v>
+      </c>
+      <c r="O687" t="n">
+        <v>0</v>
+      </c>
+      <c r="P687" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q687" t="n">
+        <v>1</v>
+      </c>
+      <c r="R687" t="n">
+        <v>2</v>
+      </c>
+      <c r="S687" t="n">
+        <v>0</v>
+      </c>
+      <c r="T687" t="n">
+        <v>0</v>
+      </c>
+      <c r="U687" t="n">
+        <v>1</v>
+      </c>
+      <c r="V687" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W687" t="n">
+        <v>30</v>
+      </c>
+      <c r="X687" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | J. GARCIA SANCHEZ | J. GODSPOWER JOHNSON | M. CAICEDO SANCHEZ | N. MC MULLEN</t>
+        </is>
+      </c>
+      <c r="D688" t="n">
+        <v>5</v>
+      </c>
+      <c r="E688" t="n">
+        <v>20</v>
+      </c>
+      <c r="F688" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G688" t="n">
+        <v>1</v>
+      </c>
+      <c r="H688" t="n">
+        <v>0</v>
+      </c>
+      <c r="I688" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J688" t="n">
+        <v>1</v>
+      </c>
+      <c r="K688" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="L688" t="n">
+        <v>0</v>
+      </c>
+      <c r="M688" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="N688" t="n">
+        <v>0</v>
+      </c>
+      <c r="O688" t="n">
+        <v>2</v>
+      </c>
+      <c r="P688" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q688" t="n">
+        <v>0</v>
+      </c>
+      <c r="R688" t="n">
+        <v>1</v>
+      </c>
+      <c r="S688" t="n">
+        <v>0</v>
+      </c>
+      <c r="T688" t="n">
+        <v>0</v>
+      </c>
+      <c r="U688" t="n">
+        <v>0</v>
+      </c>
+      <c r="V688" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W688" t="n">
+        <v>30</v>
+      </c>
+      <c r="X688" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | J. GARCIA SANCHEZ | J. GODSPOWER JOHNSON | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D689" t="n">
+        <v>5</v>
+      </c>
+      <c r="E689" t="n">
+        <v>58</v>
+      </c>
+      <c r="F689" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G689" t="n">
+        <v>6</v>
+      </c>
+      <c r="H689" t="n">
+        <v>0</v>
+      </c>
+      <c r="I689" t="n">
+        <v>2</v>
+      </c>
+      <c r="J689" t="n">
+        <v>1</v>
+      </c>
+      <c r="K689" t="n">
+        <v>300</v>
+      </c>
+      <c r="L689" t="n">
+        <v>0</v>
+      </c>
+      <c r="M689" t="n">
+        <v>300</v>
+      </c>
+      <c r="N689" t="n">
+        <v>2</v>
+      </c>
+      <c r="O689" t="n">
+        <v>0</v>
+      </c>
+      <c r="P689" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q689" t="n">
+        <v>0</v>
+      </c>
+      <c r="R689" t="n">
+        <v>1</v>
+      </c>
+      <c r="S689" t="n">
+        <v>0</v>
+      </c>
+      <c r="T689" t="n">
+        <v>0</v>
+      </c>
+      <c r="U689" t="n">
+        <v>0</v>
+      </c>
+      <c r="V689" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W689" t="n">
+        <v>30</v>
+      </c>
+      <c r="X689" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | J. GODSPOWER JOHNSON | M. CAICEDO SANCHEZ | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D690" t="n">
+        <v>5</v>
+      </c>
+      <c r="E690" t="n">
+        <v>17</v>
+      </c>
+      <c r="F690" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G690" t="n">
+        <v>1</v>
+      </c>
+      <c r="H690" t="n">
+        <v>3</v>
+      </c>
+      <c r="I690" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J690" t="n">
+        <v>1</v>
+      </c>
+      <c r="K690" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="L690" t="n">
+        <v>300</v>
+      </c>
+      <c r="M690" t="n">
+        <v>-186.36</v>
+      </c>
+      <c r="N690" t="n">
+        <v>0</v>
+      </c>
+      <c r="O690" t="n">
+        <v>2</v>
+      </c>
+      <c r="P690" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q690" t="n">
+        <v>0</v>
+      </c>
+      <c r="R690" t="n">
+        <v>2</v>
+      </c>
+      <c r="S690" t="n">
+        <v>0</v>
+      </c>
+      <c r="T690" t="n">
+        <v>0</v>
+      </c>
+      <c r="U690" t="n">
+        <v>1</v>
+      </c>
+      <c r="V690" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W690" t="n">
+        <v>30</v>
+      </c>
+      <c r="X690" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>C. DIAZ RODRIGUEZ | J. GODSPOWER JOHNSON | N. HOOVER | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D691" t="n">
+        <v>5</v>
+      </c>
+      <c r="E691" t="n">
+        <v>42</v>
+      </c>
+      <c r="F691" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G691" t="n">
+        <v>0</v>
+      </c>
+      <c r="H691" t="n">
+        <v>0</v>
+      </c>
+      <c r="I691" t="n">
+        <v>1</v>
+      </c>
+      <c r="J691" t="n">
+        <v>1</v>
+      </c>
+      <c r="K691" t="n">
+        <v>0</v>
+      </c>
+      <c r="L691" t="n">
+        <v>0</v>
+      </c>
+      <c r="M691" t="n">
+        <v>0</v>
+      </c>
+      <c r="N691" t="n">
+        <v>1</v>
+      </c>
+      <c r="O691" t="n">
+        <v>0</v>
+      </c>
+      <c r="P691" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q691" t="n">
+        <v>0</v>
+      </c>
+      <c r="R691" t="n">
+        <v>0</v>
+      </c>
+      <c r="S691" t="n">
+        <v>0</v>
+      </c>
+      <c r="T691" t="n">
+        <v>1</v>
+      </c>
+      <c r="U691" t="n">
+        <v>0</v>
+      </c>
+      <c r="V691" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W691" t="n">
+        <v>30</v>
+      </c>
+      <c r="X691" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>I. CRUZ UCEDA | J. GARCIA SANCHEZ | J. GODSPOWER JOHNSON | M. CAICEDO SANCHEZ | S. CECCARDI</t>
+        </is>
+      </c>
+      <c r="D692" t="n">
+        <v>5</v>
+      </c>
+      <c r="E692" t="n">
+        <v>49</v>
+      </c>
+      <c r="F692" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G692" t="n">
+        <v>0</v>
+      </c>
+      <c r="H692" t="n">
+        <v>4</v>
+      </c>
+      <c r="I692" t="n">
+        <v>1</v>
+      </c>
+      <c r="J692" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K692" t="n">
+        <v>0</v>
+      </c>
+      <c r="L692" t="n">
+        <v>454.55</v>
+      </c>
+      <c r="M692" t="n">
+        <v>-454.55</v>
+      </c>
+      <c r="N692" t="n">
+        <v>1</v>
+      </c>
+      <c r="O692" t="n">
+        <v>0</v>
+      </c>
+      <c r="P692" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q692" t="n">
+        <v>0</v>
+      </c>
+      <c r="R692" t="n">
+        <v>2</v>
+      </c>
+      <c r="S692" t="n">
+        <v>2</v>
+      </c>
+      <c r="T692" t="n">
+        <v>0</v>
+      </c>
+      <c r="U692" t="n">
+        <v>2</v>
+      </c>
+      <c r="V692" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W692" t="n">
+        <v>30</v>
+      </c>
+      <c r="X692" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>I. CRUZ UCEDA | M. CAICEDO SANCHEZ | M. STILMA | N. HOOVER</t>
+        </is>
+      </c>
+      <c r="D693" t="n">
+        <v>4</v>
+      </c>
+      <c r="E693" t="n">
+        <v>11</v>
+      </c>
+      <c r="F693" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G693" t="n">
+        <v>2</v>
+      </c>
+      <c r="H693" t="n">
+        <v>0</v>
+      </c>
+      <c r="I693" t="n">
+        <v>1</v>
+      </c>
+      <c r="J693" t="n">
+        <v>0</v>
+      </c>
+      <c r="K693" t="n">
+        <v>200</v>
+      </c>
+      <c r="L693" t="n">
+        <v>0</v>
+      </c>
+      <c r="M693" t="n">
+        <v>0</v>
+      </c>
+      <c r="N693" t="n">
+        <v>1</v>
+      </c>
+      <c r="O693" t="n">
+        <v>0</v>
+      </c>
+      <c r="P693" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q693" t="n">
+        <v>0</v>
+      </c>
+      <c r="R693" t="n">
+        <v>0</v>
+      </c>
+      <c r="S693" t="n">
+        <v>0</v>
+      </c>
+      <c r="T693" t="n">
+        <v>0</v>
+      </c>
+      <c r="U693" t="n">
+        <v>0</v>
+      </c>
+      <c r="V693" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W693" t="n">
+        <v>30</v>
+      </c>
+      <c r="X693" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>J. GODSPOWER JOHNSON | M. CAICEDO SANCHEZ | N. HOOVER | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D694" t="n">
+        <v>5</v>
+      </c>
+      <c r="E694" t="n">
+        <v>3</v>
+      </c>
+      <c r="F694" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G694" t="n">
+        <v>1</v>
+      </c>
+      <c r="H694" t="n">
+        <v>0</v>
+      </c>
+      <c r="I694" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J694" t="n">
+        <v>1</v>
+      </c>
+      <c r="K694" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="L694" t="n">
+        <v>0</v>
+      </c>
+      <c r="M694" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="N694" t="n">
+        <v>0</v>
+      </c>
+      <c r="O694" t="n">
+        <v>2</v>
+      </c>
+      <c r="P694" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q694" t="n">
+        <v>0</v>
+      </c>
+      <c r="R694" t="n">
+        <v>0</v>
+      </c>
+      <c r="S694" t="n">
+        <v>0</v>
+      </c>
+      <c r="T694" t="n">
+        <v>1</v>
+      </c>
+      <c r="U694" t="n">
+        <v>0</v>
+      </c>
+      <c r="V694" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W694" t="n">
+        <v>30</v>
+      </c>
+      <c r="X694" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2486526</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>J. GODSPOWER JOHNSON | M. CAICEDO SANCHEZ | P. CORDOBA MURO | S. CECCARDI | S. RODRIGUEZ FEBLES</t>
+        </is>
+      </c>
+      <c r="D695" t="n">
+        <v>5</v>
+      </c>
+      <c r="E695" t="n">
+        <v>14</v>
+      </c>
+      <c r="F695" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G695" t="n">
+        <v>2</v>
+      </c>
+      <c r="H695" t="n">
+        <v>0</v>
+      </c>
+      <c r="I695" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="J695" t="n">
+        <v>1</v>
+      </c>
+      <c r="K695" t="n">
+        <v>0</v>
+      </c>
+      <c r="L695" t="n">
+        <v>0</v>
+      </c>
+      <c r="M695" t="n">
+        <v>0</v>
+      </c>
+      <c r="N695" t="n">
+        <v>0</v>
+      </c>
+      <c r="O695" t="n">
+        <v>2</v>
+      </c>
+      <c r="P695" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q695" t="n">
+        <v>1</v>
+      </c>
+      <c r="R695" t="n">
+        <v>1</v>
+      </c>
+      <c r="S695" t="n">
+        <v>0</v>
+      </c>
+      <c r="T695" t="n">
+        <v>0</v>
+      </c>
+      <c r="U695" t="n">
+        <v>0</v>
+      </c>
+      <c r="V695" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="W695" t="n">
+        <v>30</v>
+      </c>
+      <c r="X695" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA vs MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>